<commit_message>
cpu: gate decode with issue/disp enable, rework flush priority
- decode: main inst-decode ANDs take issue_e/disp_e as an extra input,
  FU LD drivers only on disp_e; fix shorted/bunched wires in decode area
- flush: ECLR > INT > JPU/MEM priority; flush-mux E_acp, id-manager eclr,
  new inst-sfcomp (id/epoch compare). Wrong-path halt no longer fires ECLR
- todo: move finished items to the done tab, note flush priority plan

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QJGhBeyFbVexj3aLG7xNkt
</commit_message>
<xml_diff>
--- a/document/ISA-32.xlsx
+++ b/document/ISA-32.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\digital computer 32\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC7545A-122B-4856-8D43-7E9213FEE98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A1FE81-760F-45DC-BB4B-4C9A6E1649D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="211">
   <si>
     <t>opcode</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -625,10 +625,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ABI</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>return</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -842,10 +838,6 @@
   </si>
   <si>
     <t>atomize following</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>arg</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -858,12 +850,33 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>addr
-base</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>register EXT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arg, ret2</t>
+  </si>
+  <si>
+    <t>arg</t>
+  </si>
+  <si>
+    <t>at0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>at1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>addr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>kt</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ABI/alias</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1104,17 +1117,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1122,8 +1132,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1152,11 +1168,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1504,74 +1517,74 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="24"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="24"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="25"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="26"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="27"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="27"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="28"/>
-      <c r="K8" s="28"/>
-      <c r="L8" s="28"/>
-      <c r="M8" s="28"/>
-      <c r="N8" s="28"/>
-      <c r="O8" s="29"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="29"/>
+      <c r="K8" s="29"/>
+      <c r="L8" s="29"/>
+      <c r="M8" s="29"/>
+      <c r="N8" s="29"/>
+      <c r="O8" s="30"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15" t="s">
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="M9" s="15"/>
-      <c r="N9" s="15"/>
-      <c r="O9" s="16"/>
+      <c r="M9" s="20"/>
+      <c r="N9" s="20"/>
+      <c r="O9" s="21"/>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
@@ -1595,11 +1608,11 @@
       <c r="H10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="I10" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="15"/>
-      <c r="K10" s="15"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="20"/>
       <c r="L10" s="3" t="s">
         <v>46</v>
       </c>
@@ -1610,14 +1623,14 @@
         <v>91</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>147</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B11" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="20" t="s">
         <v>45</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -1635,12 +1648,12 @@
       <c r="H11" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I11" s="15" t="s">
+      <c r="I11" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15" t="s">
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20" t="s">
         <v>101</v>
       </c>
       <c r="M11" s="4" t="s">
@@ -1651,14 +1664,14 @@
         <v>gen[0]</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B12" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C12" s="15"/>
+      <c r="C12" s="20"/>
       <c r="D12" s="3" t="str">
         <f t="shared" ref="D12:D36" si="1">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D11)+1))</f>
         <v>01</v>
@@ -1675,12 +1688,12 @@
       <c r="H12" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="J12" s="15"/>
-      <c r="K12" s="15"/>
-      <c r="L12" s="15"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="20"/>
       <c r="M12" s="3" t="str">
         <f t="shared" ref="M12:M42" si="2">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M11)+1))</f>
         <v>01</v>
@@ -1689,15 +1702,15 @@
         <f t="shared" si="0"/>
         <v>gen[1]</v>
       </c>
-      <c r="O12" s="16" t="s">
-        <v>202</v>
+      <c r="O12" s="8" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B13" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C13" s="15"/>
+      <c r="C13" s="20"/>
       <c r="D13" s="3" t="str">
         <f t="shared" si="1"/>
         <v>02</v>
@@ -1708,16 +1721,16 @@
       <c r="F13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="15" t="s">
+      <c r="G13" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15" t="s">
+      <c r="H13" s="20"/>
+      <c r="I13" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="15"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
+      <c r="L13" s="20"/>
       <c r="M13" s="3" t="str">
         <f t="shared" si="2"/>
         <v>02</v>
@@ -1726,13 +1739,15 @@
         <f t="shared" si="0"/>
         <v>gen[2]</v>
       </c>
-      <c r="O13" s="16"/>
+      <c r="O13" s="21" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C14" s="15"/>
+      <c r="C14" s="20"/>
       <c r="D14" s="3" t="str">
         <f t="shared" si="1"/>
         <v>03</v>
@@ -1749,12 +1764,12 @@
       <c r="H14" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="I14" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="15"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="20"/>
+      <c r="L14" s="20"/>
       <c r="M14" s="3" t="str">
         <f t="shared" si="2"/>
         <v>03</v>
@@ -1763,13 +1778,13 @@
         <f t="shared" si="0"/>
         <v>gen[3]</v>
       </c>
-      <c r="O14" s="16"/>
+      <c r="O14" s="21"/>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C15" s="15"/>
+      <c r="C15" s="20"/>
       <c r="D15" s="3" t="str">
         <f t="shared" si="1"/>
         <v>04</v>
@@ -1786,12 +1801,12 @@
       <c r="H15" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
       <c r="M15" s="3" t="str">
         <f t="shared" si="2"/>
         <v>04</v>
@@ -1800,25 +1815,25 @@
         <f t="shared" si="0"/>
         <v>gen[4]</v>
       </c>
-      <c r="O15" s="16"/>
-      <c r="U15" s="30"/>
-      <c r="V15" s="30"/>
-      <c r="W15" s="30"/>
-      <c r="X15" s="30"/>
-      <c r="Y15" s="30"/>
-      <c r="Z15" s="30"/>
-      <c r="AA15" s="30"/>
-      <c r="AB15" s="30"/>
-      <c r="AC15" s="30"/>
-      <c r="AD15" s="30"/>
-      <c r="AF15" s="30"/>
-      <c r="AG15" s="30"/>
+      <c r="O15" s="21"/>
+      <c r="U15" s="19"/>
+      <c r="V15" s="19"/>
+      <c r="W15" s="19"/>
+      <c r="X15" s="19"/>
+      <c r="Y15" s="19"/>
+      <c r="Z15" s="19"/>
+      <c r="AA15" s="19"/>
+      <c r="AB15" s="19"/>
+      <c r="AC15" s="19"/>
+      <c r="AD15" s="19"/>
+      <c r="AF15" s="19"/>
+      <c r="AG15" s="19"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C16" s="15"/>
+      <c r="C16" s="20"/>
       <c r="D16" s="3" t="str">
         <f t="shared" si="1"/>
         <v>05</v>
@@ -1829,16 +1844,16 @@
       <c r="F16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="G16" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15" t="s">
+      <c r="H16" s="20"/>
+      <c r="I16" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="15"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="20"/>
       <c r="M16" s="3" t="str">
         <f t="shared" si="2"/>
         <v>05</v>
@@ -1847,8 +1862,8 @@
         <f t="shared" si="0"/>
         <v>gen[5]</v>
       </c>
-      <c r="O16" s="16" t="s">
-        <v>149</v>
+      <c r="O16" s="21" t="s">
+        <v>148</v>
       </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
@@ -1868,7 +1883,7 @@
       <c r="B17" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C17" s="15"/>
+      <c r="C17" s="20"/>
       <c r="D17" s="3" t="str">
         <f t="shared" si="1"/>
         <v>06</v>
@@ -1885,12 +1900,12 @@
       <c r="H17" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I17" s="15" t="s">
+      <c r="I17" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="15"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="20"/>
       <c r="M17" s="3" t="str">
         <f t="shared" si="2"/>
         <v>06</v>
@@ -1899,13 +1914,13 @@
         <f t="shared" ref="N17:N35" si="3">_xlfn.TEXTJOIN(,TRUE,"gen[",_xlfn.VALUETOTEXT(HEX2DEC(M17)),"]")</f>
         <v>gen[6]</v>
       </c>
-      <c r="O17" s="16"/>
+      <c r="O17" s="21"/>
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B18" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C18" s="15"/>
+      <c r="C18" s="20"/>
       <c r="D18" s="3" t="str">
         <f t="shared" si="1"/>
         <v>07</v>
@@ -1916,16 +1931,16 @@
       <c r="F18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="15" t="s">
+      <c r="G18" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15" t="s">
+      <c r="H18" s="20"/>
+      <c r="I18" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
+      <c r="J18" s="20"/>
+      <c r="K18" s="20"/>
+      <c r="L18" s="20"/>
       <c r="M18" s="3" t="str">
         <f t="shared" si="2"/>
         <v>07</v>
@@ -1934,14 +1949,14 @@
         <f t="shared" si="3"/>
         <v>gen[7]</v>
       </c>
-      <c r="O18" s="16"/>
+      <c r="O18" s="21"/>
       <c r="AE18" s="2"/>
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B19" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C19" s="15"/>
+      <c r="C19" s="20"/>
       <c r="D19" s="3" t="str">
         <f t="shared" si="1"/>
         <v>08</v>
@@ -1958,12 +1973,12 @@
       <c r="H19" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I19" s="15" t="s">
+      <c r="I19" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="15"/>
+      <c r="J19" s="20"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="20"/>
       <c r="M19" s="3" t="str">
         <f t="shared" si="2"/>
         <v>08</v>
@@ -1972,14 +1987,14 @@
         <f t="shared" si="3"/>
         <v>gen[8]</v>
       </c>
-      <c r="O19" s="16"/>
+      <c r="O19" s="21"/>
       <c r="V19" s="2"/>
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="15"/>
+      <c r="C20" s="20"/>
       <c r="D20" s="3" t="str">
         <f t="shared" si="1"/>
         <v>09</v>
@@ -1990,16 +2005,16 @@
       <c r="F20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="15" t="s">
+      <c r="G20" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15" t="s">
+      <c r="H20" s="20"/>
+      <c r="I20" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="15"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="20"/>
+      <c r="L20" s="20"/>
       <c r="M20" s="3" t="str">
         <f t="shared" si="2"/>
         <v>09</v>
@@ -2008,7 +2023,7 @@
         <f t="shared" si="3"/>
         <v>gen[9]</v>
       </c>
-      <c r="O20" s="16"/>
+      <c r="O20" s="21"/>
       <c r="R20" s="2"/>
       <c r="V20" s="2"/>
     </row>
@@ -2016,7 +2031,7 @@
       <c r="B21" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="15"/>
+      <c r="C21" s="20"/>
       <c r="D21" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0A</v>
@@ -2033,12 +2048,12 @@
       <c r="H21" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I21" s="15" t="s">
+      <c r="I21" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
-      <c r="L21" s="15"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="20"/>
+      <c r="L21" s="20"/>
       <c r="M21" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0A</v>
@@ -2047,13 +2062,13 @@
         <f t="shared" si="3"/>
         <v>gen[10]</v>
       </c>
-      <c r="O21" s="16"/>
+      <c r="O21" s="21"/>
     </row>
     <row r="22" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B22" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C22" s="15"/>
+      <c r="C22" s="20"/>
       <c r="D22" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0B</v>
@@ -2064,16 +2079,16 @@
       <c r="F22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="15" t="s">
+      <c r="G22" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15" t="s">
+      <c r="H22" s="20"/>
+      <c r="I22" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="20"/>
       <c r="M22" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0B</v>
@@ -2082,7 +2097,7 @@
         <f t="shared" si="3"/>
         <v>gen[11]</v>
       </c>
-      <c r="O22" s="16"/>
+      <c r="O22" s="21"/>
       <c r="S22" s="1"/>
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
@@ -2092,7 +2107,7 @@
       <c r="B23" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="15"/>
+      <c r="C23" s="20"/>
       <c r="D23" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0C</v>
@@ -2109,12 +2124,12 @@
       <c r="H23" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I23" s="15" t="s">
+      <c r="I23" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15"/>
-      <c r="L23" s="15"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
+      <c r="L23" s="20"/>
       <c r="M23" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0C</v>
@@ -2123,7 +2138,7 @@
         <f t="shared" si="3"/>
         <v>gen[12]</v>
       </c>
-      <c r="O23" s="16"/>
+      <c r="O23" s="21"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
@@ -2133,7 +2148,7 @@
       <c r="B24" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C24" s="15"/>
+      <c r="C24" s="20"/>
       <c r="D24" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0D</v>
@@ -2144,16 +2159,16 @@
       <c r="F24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="15" t="s">
+      <c r="G24" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15" t="s">
+      <c r="H24" s="20"/>
+      <c r="I24" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15"/>
-      <c r="L24" s="15"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="20"/>
+      <c r="L24" s="20"/>
       <c r="M24" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0D</v>
@@ -2162,15 +2177,15 @@
         <f t="shared" si="3"/>
         <v>gen[13]</v>
       </c>
-      <c r="O24" s="16" t="s">
-        <v>150</v>
+      <c r="O24" s="21" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C25" s="15"/>
+      <c r="C25" s="20"/>
       <c r="D25" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0E</v>
@@ -2187,12 +2202,12 @@
       <c r="H25" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I25" s="15" t="s">
+      <c r="I25" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15"/>
+      <c r="J25" s="20"/>
+      <c r="K25" s="20"/>
+      <c r="L25" s="20"/>
       <c r="M25" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0E</v>
@@ -2201,13 +2216,13 @@
         <f t="shared" si="3"/>
         <v>gen[14]</v>
       </c>
-      <c r="O25" s="16"/>
+      <c r="O25" s="21"/>
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="15"/>
+      <c r="C26" s="20"/>
       <c r="D26" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0F</v>
@@ -2218,16 +2233,16 @@
       <c r="F26" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G26" s="15" t="s">
+      <c r="G26" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15" t="s">
+      <c r="H26" s="20"/>
+      <c r="I26" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="J26" s="15"/>
-      <c r="K26" s="15"/>
-      <c r="L26" s="15"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="20"/>
+      <c r="L26" s="20"/>
       <c r="M26" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0F</v>
@@ -2236,13 +2251,13 @@
         <f t="shared" si="3"/>
         <v>gen[15]</v>
       </c>
-      <c r="O26" s="16"/>
+      <c r="O26" s="21"/>
     </row>
     <row r="27" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B27" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C27" s="15"/>
+      <c r="C27" s="20"/>
       <c r="D27" s="3" t="str">
         <f t="shared" si="1"/>
         <v>10</v>
@@ -2259,12 +2274,12 @@
       <c r="H27" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I27" s="15" t="s">
+      <c r="I27" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="J27" s="15"/>
-      <c r="K27" s="15"/>
-      <c r="L27" s="15"/>
+      <c r="J27" s="20"/>
+      <c r="K27" s="20"/>
+      <c r="L27" s="20"/>
       <c r="M27" s="3" t="str">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -2273,13 +2288,13 @@
         <f t="shared" si="3"/>
         <v>gen[16]</v>
       </c>
-      <c r="O27" s="16"/>
+      <c r="O27" s="21"/>
     </row>
     <row r="28" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B28" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C28" s="15"/>
+      <c r="C28" s="20"/>
       <c r="D28" s="3" t="str">
         <f t="shared" si="1"/>
         <v>11</v>
@@ -2296,12 +2311,12 @@
       <c r="H28" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I28" s="15" t="s">
+      <c r="I28" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="J28" s="15"/>
-      <c r="K28" s="15"/>
-      <c r="L28" s="15"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
+      <c r="L28" s="20"/>
       <c r="M28" s="3" t="str">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -2310,13 +2325,13 @@
         <f t="shared" si="3"/>
         <v>gen[17]</v>
       </c>
-      <c r="O28" s="16"/>
+      <c r="O28" s="21"/>
     </row>
     <row r="29" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B29" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C29" s="15"/>
+      <c r="C29" s="20"/>
       <c r="D29" s="3" t="str">
         <f t="shared" si="1"/>
         <v>12</v>
@@ -2327,16 +2342,16 @@
       <c r="F29" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G29" s="15" t="s">
+      <c r="G29" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15" t="s">
+      <c r="H29" s="20"/>
+      <c r="I29" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="J29" s="15"/>
-      <c r="K29" s="15"/>
-      <c r="L29" s="15"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="20"/>
+      <c r="L29" s="20"/>
       <c r="M29" s="3" t="str">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -2345,13 +2360,13 @@
         <f t="shared" si="3"/>
         <v>gen[18]</v>
       </c>
-      <c r="O29" s="16"/>
+      <c r="O29" s="21"/>
     </row>
     <row r="30" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B30" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C30" s="15"/>
+      <c r="C30" s="20"/>
       <c r="D30" s="3" t="str">
         <f t="shared" si="1"/>
         <v>13</v>
@@ -2368,12 +2383,12 @@
       <c r="H30" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I30" s="15" t="s">
+      <c r="I30" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="J30" s="15"/>
-      <c r="K30" s="15"/>
-      <c r="L30" s="15"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="20"/>
+      <c r="L30" s="20"/>
       <c r="M30" s="3" t="str">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -2382,13 +2397,13 @@
         <f t="shared" si="3"/>
         <v>gen[19]</v>
       </c>
-      <c r="O30" s="16"/>
+      <c r="O30" s="21"/>
     </row>
     <row r="31" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B31" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C31" s="15"/>
+      <c r="C31" s="20"/>
       <c r="D31" s="3" t="str">
         <f t="shared" si="1"/>
         <v>14</v>
@@ -2405,12 +2420,12 @@
       <c r="H31" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I31" s="15" t="s">
+      <c r="I31" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="J31" s="15"/>
-      <c r="K31" s="15"/>
-      <c r="L31" s="15"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="20"/>
       <c r="M31" s="3" t="str">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -2419,13 +2434,13 @@
         <f t="shared" si="3"/>
         <v>gen[20]</v>
       </c>
-      <c r="O31" s="16"/>
+      <c r="O31" s="21"/>
     </row>
     <row r="32" spans="2:31" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C32" s="15"/>
+      <c r="C32" s="20"/>
       <c r="D32" s="3" t="str">
         <f t="shared" si="1"/>
         <v>15</v>
@@ -2436,16 +2451,16 @@
       <c r="F32" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G32" s="15" t="s">
+      <c r="G32" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H32" s="15"/>
-      <c r="I32" s="15" t="s">
+      <c r="H32" s="20"/>
+      <c r="I32" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="J32" s="15"/>
-      <c r="K32" s="15"/>
-      <c r="L32" s="15"/>
+      <c r="J32" s="20"/>
+      <c r="K32" s="20"/>
+      <c r="L32" s="20"/>
       <c r="M32" s="3" t="str">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -2454,15 +2469,15 @@
         <f t="shared" si="3"/>
         <v>gen[21]</v>
       </c>
-      <c r="O32" s="20" t="s">
-        <v>205</v>
+      <c r="O32" s="8" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B33" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C33" s="15"/>
+      <c r="C33" s="20"/>
       <c r="D33" s="3" t="str">
         <f t="shared" si="1"/>
         <v>16</v>
@@ -2479,12 +2494,12 @@
       <c r="H33" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I33" s="15" t="s">
+      <c r="I33" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="J33" s="15"/>
-      <c r="K33" s="15"/>
-      <c r="L33" s="15"/>
+      <c r="J33" s="20"/>
+      <c r="K33" s="20"/>
+      <c r="L33" s="20"/>
       <c r="M33" s="3" t="str">
         <f t="shared" si="2"/>
         <v>16</v>
@@ -2493,13 +2508,15 @@
         <f t="shared" si="3"/>
         <v>gen[22]</v>
       </c>
-      <c r="O33" s="16"/>
+      <c r="O33" s="8" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="34" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B34" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C34" s="15"/>
+      <c r="C34" s="20"/>
       <c r="D34" s="3" t="str">
         <f t="shared" si="1"/>
         <v>17</v>
@@ -2510,16 +2527,16 @@
       <c r="F34" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="15" t="s">
+      <c r="G34" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H34" s="15"/>
-      <c r="I34" s="15" t="s">
+      <c r="H34" s="20"/>
+      <c r="I34" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="J34" s="15"/>
-      <c r="K34" s="15"/>
-      <c r="L34" s="15"/>
+      <c r="J34" s="20"/>
+      <c r="K34" s="20"/>
+      <c r="L34" s="20"/>
       <c r="M34" s="3" t="str">
         <f t="shared" si="2"/>
         <v>17</v>
@@ -2528,22 +2545,24 @@
         <f t="shared" si="3"/>
         <v>gen[23]</v>
       </c>
-      <c r="O34" s="16"/>
+      <c r="O34" s="8" t="s">
+        <v>209</v>
+      </c>
       <c r="R34" t="s">
         <v>136</v>
       </c>
-      <c r="T34" s="30"/>
-      <c r="U34" s="30"/>
-      <c r="V34" s="30"/>
-      <c r="W34" s="30"/>
-      <c r="X34" s="30"/>
-      <c r="Y34" s="30"/>
+      <c r="T34" s="19"/>
+      <c r="U34" s="19"/>
+      <c r="V34" s="19"/>
+      <c r="W34" s="19"/>
+      <c r="X34" s="19"/>
+      <c r="Y34" s="19"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C35" s="15"/>
+      <c r="C35" s="20"/>
       <c r="D35" s="3" t="str">
         <f t="shared" si="1"/>
         <v>18</v>
@@ -2560,12 +2579,12 @@
       <c r="H35" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I35" s="15" t="s">
+      <c r="I35" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="J35" s="15"/>
-      <c r="K35" s="15"/>
-      <c r="L35" s="15"/>
+      <c r="J35" s="20"/>
+      <c r="K35" s="20"/>
+      <c r="L35" s="20"/>
       <c r="M35" s="3" t="str">
         <f t="shared" si="2"/>
         <v>18</v>
@@ -2574,19 +2593,21 @@
         <f t="shared" si="3"/>
         <v>gen[24]</v>
       </c>
-      <c r="O35" s="16"/>
-      <c r="T35" s="30"/>
-      <c r="U35" s="30"/>
-      <c r="V35" s="30"/>
-      <c r="W35" s="30"/>
-      <c r="X35" s="30"/>
-      <c r="Y35" s="30"/>
+      <c r="O35" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="T35" s="19"/>
+      <c r="U35" s="19"/>
+      <c r="V35" s="19"/>
+      <c r="W35" s="19"/>
+      <c r="X35" s="19"/>
+      <c r="Y35" s="19"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C36" s="15"/>
+      <c r="C36" s="20"/>
       <c r="D36" s="3" t="str">
         <f t="shared" si="1"/>
         <v>19</v>
@@ -2597,16 +2618,16 @@
       <c r="F36" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="15" t="s">
+      <c r="G36" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H36" s="15"/>
-      <c r="I36" s="15" t="s">
+      <c r="H36" s="20"/>
+      <c r="I36" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="J36" s="15"/>
-      <c r="K36" s="15"/>
-      <c r="L36" s="15"/>
+      <c r="J36" s="20"/>
+      <c r="K36" s="20"/>
+      <c r="L36" s="20"/>
       <c r="M36" s="3" t="str">
         <f t="shared" si="2"/>
         <v>19</v>
@@ -2622,7 +2643,7 @@
       <c r="B37" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="15" t="s">
+      <c r="C37" s="20" t="s">
         <v>47</v>
       </c>
       <c r="D37" s="3" t="str">
@@ -2635,16 +2656,16 @@
       <c r="F37" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G37" s="15" t="s">
+      <c r="G37" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H37" s="15"/>
-      <c r="I37" s="15" t="s">
+      <c r="H37" s="20"/>
+      <c r="I37" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="J37" s="15"/>
-      <c r="K37" s="15"/>
-      <c r="L37" s="15" t="s">
+      <c r="J37" s="20"/>
+      <c r="K37" s="20"/>
+      <c r="L37" s="20" t="s">
         <v>102</v>
       </c>
       <c r="M37" s="3" t="str">
@@ -2654,7 +2675,7 @@
       <c r="N37" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="O37" s="16" t="s">
+      <c r="O37" s="21" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2662,7 +2683,7 @@
       <c r="B38" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C38" s="15"/>
+      <c r="C38" s="20"/>
       <c r="D38" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1B</v>
@@ -2673,16 +2694,16 @@
       <c r="F38" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G38" s="15" t="s">
+      <c r="G38" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H38" s="15"/>
-      <c r="I38" s="15" t="s">
+      <c r="H38" s="20"/>
+      <c r="I38" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="J38" s="15"/>
-      <c r="K38" s="15"/>
-      <c r="L38" s="15"/>
+      <c r="J38" s="20"/>
+      <c r="K38" s="20"/>
+      <c r="L38" s="20"/>
       <c r="M38" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1B</v>
@@ -2690,13 +2711,13 @@
       <c r="N38" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="16"/>
+      <c r="O38" s="21"/>
     </row>
     <row r="39" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B39" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C39" s="15"/>
+      <c r="C39" s="20"/>
       <c r="D39" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1C</v>
@@ -2713,12 +2734,12 @@
       <c r="H39" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I39" s="15" t="s">
+      <c r="I39" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="J39" s="15"/>
-      <c r="K39" s="15"/>
-      <c r="L39" s="15"/>
+      <c r="J39" s="20"/>
+      <c r="K39" s="20"/>
+      <c r="L39" s="20"/>
       <c r="M39" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1C</v>
@@ -2726,7 +2747,7 @@
       <c r="N39" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O39" s="16"/>
+      <c r="O39" s="21"/>
     </row>
     <row r="40" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B40" s="9" t="s">
@@ -2742,16 +2763,16 @@
       <c r="E40" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="F40" s="15" t="s">
+      <c r="F40" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G40" s="15"/>
-      <c r="H40" s="15"/>
-      <c r="I40" s="15" t="s">
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="J40" s="15"/>
-      <c r="K40" s="15"/>
+      <c r="J40" s="20"/>
+      <c r="K40" s="20"/>
       <c r="L40" s="5" t="s">
         <v>103</v>
       </c>
@@ -2762,15 +2783,15 @@
       <c r="N40" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O40" s="16" t="s">
-        <v>163</v>
+      <c r="O40" s="21" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="41" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B41" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C41" s="15" t="s">
+      <c r="C41" s="20" t="s">
         <v>3</v>
       </c>
       <c r="D41" s="3" t="str">
@@ -2783,15 +2804,15 @@
       <c r="F41" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G41" s="15" t="s">
+      <c r="G41" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="H41" s="15"/>
-      <c r="I41" s="15" t="s">
+      <c r="H41" s="20"/>
+      <c r="I41" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="J41" s="15"/>
-      <c r="K41" s="15"/>
+      <c r="J41" s="20"/>
+      <c r="K41" s="20"/>
       <c r="L41" s="5" t="s">
         <v>104</v>
       </c>
@@ -2802,14 +2823,14 @@
       <c r="N41" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="O41" s="16"/>
+      <c r="O41" s="21"/>
       <c r="T41" s="2"/>
     </row>
     <row r="42" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B42" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C42" s="15"/>
+      <c r="C42" s="20"/>
       <c r="D42" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1F</v>
@@ -2820,15 +2841,15 @@
       <c r="F42" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G42" s="15" t="s">
+      <c r="G42" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="H42" s="15"/>
-      <c r="I42" s="15" t="s">
+      <c r="H42" s="20"/>
+      <c r="I42" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="J42" s="15"/>
-      <c r="K42" s="15"/>
+      <c r="J42" s="20"/>
+      <c r="K42" s="20"/>
       <c r="L42" s="5" t="s">
         <v>104</v>
       </c>
@@ -2839,13 +2860,13 @@
       <c r="N42" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="O42" s="16"/>
+      <c r="O42" s="21"/>
     </row>
     <row r="43" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B43" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C43" s="15" t="s">
+      <c r="C43" s="20" t="s">
         <v>51</v>
       </c>
       <c r="D43" s="3" t="str">
@@ -2858,27 +2879,27 @@
       <c r="F43" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G43" s="15" t="s">
+      <c r="G43" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="H43" s="15"/>
-      <c r="I43" s="15" t="s">
+      <c r="H43" s="20"/>
+      <c r="I43" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="J43" s="15"/>
-      <c r="K43" s="15"/>
-      <c r="L43" s="15" t="s">
+      <c r="J43" s="20"/>
+      <c r="K43" s="20"/>
+      <c r="L43" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="M43" s="15"/>
-      <c r="N43" s="15"/>
-      <c r="O43" s="16"/>
+      <c r="M43" s="20"/>
+      <c r="N43" s="20"/>
+      <c r="O43" s="21"/>
     </row>
     <row r="44" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B44" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C44" s="15"/>
+      <c r="C44" s="20"/>
       <c r="D44" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 32))</f>
         <v>40~5F</v>
@@ -2889,31 +2910,31 @@
       <c r="F44" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G44" s="15" t="s">
+      <c r="G44" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="H44" s="15"/>
-      <c r="I44" s="15" t="s">
+      <c r="H44" s="20"/>
+      <c r="I44" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="J44" s="15"/>
-      <c r="K44" s="15"/>
+      <c r="J44" s="20"/>
+      <c r="K44" s="20"/>
       <c r="L44" s="6" t="s">
         <v>46</v>
       </c>
       <c r="M44" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="N44" s="15" t="s">
+      <c r="N44" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="O44" s="16"/>
+      <c r="O44" s="21"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B45" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C45" s="15" t="s">
+      <c r="C45" s="20" t="s">
         <v>52</v>
       </c>
       <c r="D45" s="3" t="str">
@@ -2926,31 +2947,31 @@
       <c r="F45" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G45" s="15" t="s">
+      <c r="G45" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="H45" s="15"/>
-      <c r="I45" s="15" t="s">
+      <c r="H45" s="20"/>
+      <c r="I45" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="J45" s="15"/>
-      <c r="K45" s="15"/>
+      <c r="J45" s="20"/>
+      <c r="K45" s="20"/>
       <c r="L45" s="5" t="s">
         <v>105</v>
       </c>
       <c r="M45" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="N45" s="15" t="s">
+      <c r="N45" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="O45" s="16"/>
+      <c r="O45" s="21"/>
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B46" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C46" s="15"/>
+      <c r="C46" s="20"/>
       <c r="D46" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 8))</f>
         <v>68~6F</v>
@@ -2961,15 +2982,15 @@
       <c r="F46" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G46" s="15" t="s">
+      <c r="G46" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="H46" s="15"/>
-      <c r="I46" s="15" t="s">
+      <c r="H46" s="20"/>
+      <c r="I46" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="J46" s="15"/>
-      <c r="K46" s="15"/>
+      <c r="J46" s="20"/>
+      <c r="K46" s="20"/>
       <c r="L46" s="5" t="s">
         <v>105</v>
       </c>
@@ -2977,16 +2998,16 @@
         <f t="shared" ref="M46:M52" si="5">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M45)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M45)+1))</f>
         <v>01</v>
       </c>
-      <c r="N46" s="15" t="s">
+      <c r="N46" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="O46" s="16"/>
+      <c r="O46" s="21"/>
     </row>
     <row r="47" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B47" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C47" s="15"/>
+      <c r="C47" s="20"/>
       <c r="D47" s="4" t="str">
         <f>DEC2HEX(HEX2DEC(RIGHT(D46,LEN(D46)-FIND("~",D46,1))) + 1)</f>
         <v>70</v>
@@ -2997,15 +3018,15 @@
       <c r="F47" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G47" s="15" t="s">
+      <c r="G47" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="H47" s="15"/>
-      <c r="I47" s="15" t="s">
+      <c r="H47" s="20"/>
+      <c r="I47" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="J47" s="15"/>
-      <c r="K47" s="15"/>
+      <c r="J47" s="20"/>
+      <c r="K47" s="20"/>
       <c r="L47" s="5" t="s">
         <v>105</v>
       </c>
@@ -3013,16 +3034,16 @@
         <f t="shared" si="5"/>
         <v>02</v>
       </c>
-      <c r="N47" s="15" t="s">
+      <c r="N47" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="O47" s="16"/>
+      <c r="O47" s="21"/>
     </row>
     <row r="48" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B48" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C48" s="15"/>
+      <c r="C48" s="20"/>
       <c r="D48" s="3" t="str">
         <f t="shared" ref="D48:D54" si="6">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D47)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D47)+1))</f>
         <v>71</v>
@@ -3030,16 +3051,16 @@
       <c r="E48" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F48" s="15" t="s">
+      <c r="F48" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G48" s="15"/>
-      <c r="H48" s="15"/>
-      <c r="I48" s="15" t="s">
+      <c r="G48" s="20"/>
+      <c r="H48" s="20"/>
+      <c r="I48" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="J48" s="15"/>
-      <c r="K48" s="15"/>
+      <c r="J48" s="20"/>
+      <c r="K48" s="20"/>
       <c r="L48" s="5" t="s">
         <v>107</v>
       </c>
@@ -3047,16 +3068,16 @@
         <f t="shared" si="5"/>
         <v>03</v>
       </c>
-      <c r="N48" s="15" t="s">
+      <c r="N48" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="O48" s="16"/>
+      <c r="O48" s="21"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C49" s="15"/>
+      <c r="C49" s="20"/>
       <c r="D49" s="3" t="str">
         <f t="shared" si="6"/>
         <v>72</v>
@@ -3064,16 +3085,16 @@
       <c r="E49" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F49" s="15" t="s">
+      <c r="F49" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G49" s="15"/>
-      <c r="H49" s="15"/>
-      <c r="I49" s="15" t="s">
+      <c r="G49" s="20"/>
+      <c r="H49" s="20"/>
+      <c r="I49" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="J49" s="15"/>
-      <c r="K49" s="15"/>
+      <c r="J49" s="20"/>
+      <c r="K49" s="20"/>
       <c r="L49" s="5" t="s">
         <v>105</v>
       </c>
@@ -3081,33 +3102,33 @@
         <f t="shared" si="5"/>
         <v>04</v>
       </c>
-      <c r="N49" s="15" t="s">
+      <c r="N49" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="O49" s="16"/>
+      <c r="O49" s="21"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C50" s="15"/>
+      <c r="C50" s="20"/>
       <c r="D50" s="3" t="str">
         <f t="shared" si="6"/>
         <v>73</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="F50" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="F50" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G50" s="15"/>
-      <c r="H50" s="15"/>
-      <c r="I50" s="15" t="s">
-        <v>175</v>
-      </c>
-      <c r="J50" s="15"/>
-      <c r="K50" s="15"/>
+      <c r="G50" s="20"/>
+      <c r="H50" s="20"/>
+      <c r="I50" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="J50" s="20"/>
+      <c r="K50" s="20"/>
       <c r="L50" s="5" t="s">
         <v>105</v>
       </c>
@@ -3115,33 +3136,33 @@
         <f t="shared" si="5"/>
         <v>05</v>
       </c>
-      <c r="N50" s="15" t="s">
+      <c r="N50" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="O50" s="16"/>
+      <c r="O50" s="21"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C51" s="15"/>
+      <c r="C51" s="20"/>
       <c r="D51" s="3" t="str">
         <f t="shared" si="6"/>
         <v>74</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="F51" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="F51" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G51" s="15"/>
-      <c r="H51" s="15"/>
-      <c r="I51" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="J51" s="15"/>
-      <c r="K51" s="15"/>
+      <c r="G51" s="20"/>
+      <c r="H51" s="20"/>
+      <c r="I51" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="J51" s="20"/>
+      <c r="K51" s="20"/>
       <c r="L51" s="5" t="s">
         <v>108</v>
       </c>
@@ -3149,16 +3170,16 @@
         <f t="shared" si="5"/>
         <v>06</v>
       </c>
-      <c r="N51" s="15" t="s">
+      <c r="N51" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="O51" s="16"/>
+      <c r="O51" s="21"/>
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C52" s="15"/>
+      <c r="C52" s="20"/>
       <c r="D52" s="3" t="str">
         <f t="shared" si="6"/>
         <v>75</v>
@@ -3166,16 +3187,16 @@
       <c r="E52" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F52" s="15" t="s">
+      <c r="F52" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G52" s="15"/>
-      <c r="H52" s="15"/>
-      <c r="I52" s="15" t="s">
+      <c r="G52" s="20"/>
+      <c r="H52" s="20"/>
+      <c r="I52" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="J52" s="15"/>
-      <c r="K52" s="15"/>
+      <c r="J52" s="20"/>
+      <c r="K52" s="20"/>
       <c r="L52" s="5" t="s">
         <v>107</v>
       </c>
@@ -3183,16 +3204,16 @@
         <f t="shared" si="5"/>
         <v>07</v>
       </c>
-      <c r="N52" s="15" t="s">
+      <c r="N52" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="O52" s="16"/>
+      <c r="O52" s="21"/>
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C53" s="15" t="s">
+      <c r="C53" s="20" t="s">
         <v>50</v>
       </c>
       <c r="D53" s="3" t="str">
@@ -3202,16 +3223,16 @@
       <c r="E53" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="F53" s="15" t="s">
+      <c r="F53" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G53" s="15"/>
-      <c r="H53" s="15"/>
-      <c r="I53" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="J53" s="15"/>
-      <c r="K53" s="15"/>
+      <c r="G53" s="20"/>
+      <c r="H53" s="20"/>
+      <c r="I53" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="J53" s="20"/>
+      <c r="K53" s="20"/>
       <c r="L53" s="5" t="s">
         <v>107</v>
       </c>
@@ -3219,16 +3240,16 @@
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(M52) + 1),"~",DEC2HEX(HEX2DEC(M52) + 6))</f>
         <v>8~D</v>
       </c>
-      <c r="N53" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="O53" s="16"/>
+      <c r="N53" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="O53" s="21"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C54" s="15"/>
+      <c r="C54" s="20"/>
       <c r="D54" s="3" t="str">
         <f t="shared" si="6"/>
         <v>77</v>
@@ -3236,16 +3257,16 @@
       <c r="E54" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F54" s="15" t="s">
+      <c r="F54" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G54" s="15"/>
-      <c r="H54" s="15"/>
-      <c r="I54" s="15" t="s">
+      <c r="G54" s="20"/>
+      <c r="H54" s="20"/>
+      <c r="I54" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="J54" s="15"/>
-      <c r="K54" s="15"/>
+      <c r="J54" s="20"/>
+      <c r="K54" s="20"/>
       <c r="L54" s="5" t="s">
         <v>107</v>
       </c>
@@ -3253,16 +3274,16 @@
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(M53,LEN(M53)-FIND("~",M53,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(M53,LEN(M53)-FIND("~",M53,1))) + 16))</f>
         <v>E~1D</v>
       </c>
-      <c r="N54" s="15" t="s">
+      <c r="N54" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="O54" s="16"/>
+      <c r="O54" s="21"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C55" s="15"/>
+      <c r="C55" s="20"/>
       <c r="D55" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D54)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D54)+1))</f>
         <v>78</v>
@@ -3274,49 +3295,49 @@
         <v>4</v>
       </c>
       <c r="G55" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="I55" s="20" t="s">
         <v>152</v>
       </c>
-      <c r="H55" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="I55" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="J55" s="15"/>
-      <c r="K55" s="15"/>
-      <c r="L55" s="15" t="s">
+      <c r="J55" s="20"/>
+      <c r="K55" s="20"/>
+      <c r="L55" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="M55" s="15"/>
-      <c r="N55" s="15"/>
-      <c r="O55" s="16"/>
+      <c r="M55" s="20"/>
+      <c r="N55" s="20"/>
+      <c r="O55" s="21"/>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C56" s="15"/>
+      <c r="C56" s="20"/>
       <c r="D56" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D55)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D55)+1))</f>
         <v>79</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>92</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="I56" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="J56" s="15"/>
-      <c r="K56" s="15"/>
+      <c r="I56" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="J56" s="20"/>
+      <c r="K56" s="20"/>
       <c r="L56" s="5" t="s">
         <v>39</v>
       </c>
@@ -3334,7 +3355,7 @@
       <c r="B57" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C57" s="15" t="s">
+      <c r="C57" s="20" t="s">
         <v>47</v>
       </c>
       <c r="D57" s="3" t="str">
@@ -3342,7 +3363,7 @@
         <v>7A</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>11</v>
@@ -3351,13 +3372,13 @@
         <v>92</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="I57" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="J57" s="15"/>
-      <c r="K57" s="15"/>
+        <v>193</v>
+      </c>
+      <c r="I57" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="J57" s="20"/>
+      <c r="K57" s="20"/>
       <c r="L57" s="4" t="s">
         <v>96</v>
       </c>
@@ -3376,13 +3397,13 @@
       <c r="B58" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C58" s="15"/>
+      <c r="C58" s="20"/>
       <c r="D58" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D57)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D57)+1))</f>
         <v>7B</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>12</v>
@@ -3391,13 +3412,13 @@
         <v>92</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="I58" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="J58" s="15"/>
-      <c r="K58" s="15"/>
+        <v>193</v>
+      </c>
+      <c r="I58" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="J58" s="20"/>
+      <c r="K58" s="20"/>
       <c r="L58" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L57+1)</f>
         <v>1</v>
@@ -3417,7 +3438,7 @@
       <c r="B59" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C59" s="15" t="s">
+      <c r="C59" s="20" t="s">
         <v>38</v>
       </c>
       <c r="D59" s="3" t="str">
@@ -3425,20 +3446,20 @@
         <v>7C</v>
       </c>
       <c r="E59" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="F59" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="G59" s="20"/>
+      <c r="H59" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="F59" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="G59" s="15"/>
-      <c r="H59" s="3" t="s">
+      <c r="I59" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="I59" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="J59" s="15"/>
-      <c r="K59" s="15"/>
+      <c r="J59" s="20"/>
+      <c r="K59" s="20"/>
       <c r="L59" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L58+1)</f>
         <v>2</v>
@@ -3458,28 +3479,28 @@
       <c r="B60" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C60" s="15"/>
+      <c r="C60" s="20"/>
       <c r="D60" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7D</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F60" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G60" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G60" s="3" t="s">
+      <c r="H60" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="H60" s="3" t="s">
+      <c r="I60" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="I60" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="J60" s="15"/>
-      <c r="K60" s="15"/>
+      <c r="J60" s="20"/>
+      <c r="K60" s="20"/>
       <c r="L60" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L59+1)</f>
         <v>3</v>
@@ -3510,57 +3531,57 @@
         <v>82</v>
       </c>
       <c r="F61" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="G61" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="G61" s="13" t="s">
-        <v>173</v>
-      </c>
       <c r="H61" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="I61" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="J61" s="15"/>
-      <c r="K61" s="15"/>
-      <c r="L61" s="14" t="s">
-        <v>206</v>
-      </c>
-      <c r="M61" s="14"/>
-      <c r="N61" s="14"/>
-      <c r="O61" s="20"/>
+        <v>170</v>
+      </c>
+      <c r="I61" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="J61" s="20"/>
+      <c r="K61" s="20"/>
+      <c r="L61" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="M61" s="15"/>
+      <c r="N61" s="15"/>
+      <c r="O61" s="16"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="9" t="s">
         <v>90</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7F</v>
       </c>
       <c r="E62" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F62" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="G62" s="20"/>
+      <c r="H62" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="F62" s="15" t="s">
+      <c r="I62" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="G62" s="15"/>
-      <c r="H62" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="I62" s="15" t="s">
-        <v>201</v>
-      </c>
-      <c r="J62" s="15"/>
-      <c r="K62" s="15"/>
+      <c r="J62" s="20"/>
+      <c r="K62" s="20"/>
       <c r="L62" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M62" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="N62" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L67,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L67,"-", -1))+1,"0"))</f>
@@ -3573,7 +3594,7 @@
         <v>90</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(D62) + 1),"~","FF")</f>
@@ -3582,22 +3603,22 @@
       <c r="E63" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F63" s="15" t="s">
+      <c r="F63" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G63" s="15"/>
-      <c r="H63" s="15"/>
-      <c r="I63" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="J63" s="15"/>
-      <c r="K63" s="15"/>
+      <c r="G63" s="20"/>
+      <c r="H63" s="20"/>
+      <c r="I63" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="J63" s="20"/>
+      <c r="K63" s="20"/>
       <c r="L63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L62,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L62,"-", -1))+1,"0"))</f>
         <v>ex-2</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N62,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N62,"-", -1))+1,"0"))</f>
@@ -3606,32 +3627,32 @@
       <c r="O63" s="10"/>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B64" s="18" t="s">
+      <c r="B64" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="E64" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="C64" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="E64" s="3" t="s">
+      <c r="F64" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="F64" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="G64" s="15"/>
-      <c r="H64" s="15"/>
-      <c r="I64" s="15"/>
-      <c r="J64" s="15"/>
-      <c r="K64" s="15"/>
+      <c r="G64" s="20"/>
+      <c r="H64" s="20"/>
+      <c r="I64" s="20"/>
+      <c r="J64" s="20"/>
+      <c r="K64" s="20"/>
       <c r="L64" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L63,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L63,"-", -1))+1,"0"))</f>
         <v>ex-3</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="N64" s="3" t="str">
         <f t="shared" ref="N64:N67" si="8">_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N63,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N63,"-", -1))+1,"0"))</f>
@@ -3640,30 +3661,30 @@
       <c r="O64" s="10"/>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B65" s="18"/>
+      <c r="B65" s="17"/>
       <c r="C65" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D65" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E65" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="F65" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="F65" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G65" s="15"/>
-      <c r="H65" s="15"/>
-      <c r="I65" s="15"/>
-      <c r="J65" s="15"/>
-      <c r="K65" s="15"/>
+      <c r="G65" s="20"/>
+      <c r="H65" s="20"/>
+      <c r="I65" s="20"/>
+      <c r="J65" s="20"/>
+      <c r="K65" s="20"/>
       <c r="L65" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L64,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L64,"-", -1))+1,"0"))</f>
         <v>ex-4</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N65" s="3" t="str">
         <f t="shared" si="8"/>
@@ -3672,24 +3693,24 @@
       <c r="O65" s="10"/>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B66" s="18"/>
-      <c r="C66" s="14" t="s">
-        <v>204</v>
-      </c>
-      <c r="D66" s="15"/>
-      <c r="E66" s="15"/>
-      <c r="F66" s="15"/>
-      <c r="G66" s="15"/>
-      <c r="H66" s="15"/>
-      <c r="I66" s="15"/>
-      <c r="J66" s="15"/>
-      <c r="K66" s="15"/>
+      <c r="B66" s="17"/>
+      <c r="C66" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="20"/>
+      <c r="I66" s="20"/>
+      <c r="J66" s="20"/>
+      <c r="K66" s="20"/>
       <c r="L66" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L65,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L65,"-", -1))+1,"0"))</f>
         <v>ex-5</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="N66" s="3" t="str">
         <f t="shared" si="8"/>
@@ -3698,31 +3719,134 @@
       <c r="O66" s="10"/>
     </row>
     <row r="67" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B67" s="19"/>
-      <c r="C67" s="17"/>
-      <c r="D67" s="17"/>
-      <c r="E67" s="17"/>
-      <c r="F67" s="17"/>
-      <c r="G67" s="17"/>
-      <c r="H67" s="17"/>
-      <c r="I67" s="17"/>
-      <c r="J67" s="17"/>
-      <c r="K67" s="17"/>
+      <c r="B67" s="18"/>
+      <c r="C67" s="31"/>
+      <c r="D67" s="31"/>
+      <c r="E67" s="31"/>
+      <c r="F67" s="31"/>
+      <c r="G67" s="31"/>
+      <c r="H67" s="31"/>
+      <c r="I67" s="31"/>
+      <c r="J67" s="31"/>
+      <c r="K67" s="31"/>
       <c r="L67" s="12" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L66,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L66,"-", -1))+1,"0"))</f>
         <v>ex-6</v>
       </c>
       <c r="M67" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="N67" s="12" t="str">
         <f t="shared" si="8"/>
         <v>ex-12</v>
       </c>
-      <c r="O67" s="31"/>
+      <c r="O67" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="128">
+  <mergeCells count="127">
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="N46:O46"/>
+    <mergeCell ref="N47:O47"/>
+    <mergeCell ref="N48:O48"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="C66:F67"/>
+    <mergeCell ref="G64:K67"/>
+    <mergeCell ref="I61:K61"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="O40:O42"/>
+    <mergeCell ref="F63:H63"/>
+    <mergeCell ref="I63:K63"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="N53:O53"/>
+    <mergeCell ref="N54:O54"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="I59:K59"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="L55:O55"/>
+    <mergeCell ref="F54:H54"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="F53:H53"/>
+    <mergeCell ref="C53:C56"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="B6:O8"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="O16:O23"/>
+    <mergeCell ref="O24:O31"/>
+    <mergeCell ref="L11:L36"/>
+    <mergeCell ref="C11:C36"/>
+    <mergeCell ref="O13:O15"/>
+    <mergeCell ref="C45:C52"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="F51:H51"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="N44:O44"/>
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:K46"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="O37:O39"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
     <mergeCell ref="L61:O61"/>
     <mergeCell ref="B64:B67"/>
     <mergeCell ref="AF15:AG15"/>
@@ -3747,110 +3871,6 @@
     <mergeCell ref="G36:H36"/>
     <mergeCell ref="U15:AB15"/>
     <mergeCell ref="I55:K55"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="N44:O44"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="C45:C52"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="B6:O8"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="O16:O23"/>
-    <mergeCell ref="O24:O31"/>
-    <mergeCell ref="L11:L36"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="O12:O15"/>
-    <mergeCell ref="O32:O35"/>
-    <mergeCell ref="O37:O39"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="N46:O46"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="N48:O48"/>
-    <mergeCell ref="N49:O49"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="C66:F67"/>
-    <mergeCell ref="G64:K67"/>
-    <mergeCell ref="I61:K61"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="O40:O42"/>
-    <mergeCell ref="F63:H63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="N53:O53"/>
-    <mergeCell ref="N54:O54"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="L55:O55"/>
-    <mergeCell ref="F54:H54"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="F53:H53"/>
-    <mergeCell ref="C53:C56"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="F62:G62"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
cpu[chore]: wire rework for interrupt sequencer
</commit_message>
<xml_diff>
--- a/document/ISA-32.xlsx
+++ b/document/ISA-32.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\digital computer 32\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A1FE81-760F-45DC-BB4B-4C9A6E1649D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D6B8DB9-B1DF-459F-A3DF-A52E944852A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
+    <workbookView xWindow="7380" yWindow="675" windowWidth="28800" windowHeight="12915" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -625,10 +625,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>return</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>callee</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -854,9 +850,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>arg, ret2</t>
-  </si>
-  <si>
     <t>arg</t>
   </si>
   <si>
@@ -877,6 +870,14 @@
   </si>
   <si>
     <t>ABI/alias</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>return,lret</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arg,hret</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1623,7 +1624,7 @@
         <v>91</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
@@ -1664,7 +1665,7 @@
         <v>gen[0]</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>147</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
@@ -1703,7 +1704,7 @@
         <v>gen[1]</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
@@ -1740,7 +1741,7 @@
         <v>gen[2]</v>
       </c>
       <c r="O13" s="21" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
@@ -1863,7 +1864,7 @@
         <v>gen[5]</v>
       </c>
       <c r="O16" s="21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
@@ -2178,7 +2179,7 @@
         <v>gen[13]</v>
       </c>
       <c r="O24" s="21" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.3">
@@ -2470,7 +2471,7 @@
         <v>gen[21]</v>
       </c>
       <c r="O32" s="8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.3">
@@ -2509,7 +2510,7 @@
         <v>gen[22]</v>
       </c>
       <c r="O33" s="8" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="34" spans="2:25" x14ac:dyDescent="0.3">
@@ -2546,7 +2547,7 @@
         <v>gen[23]</v>
       </c>
       <c r="O34" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="R34" t="s">
         <v>136</v>
@@ -2594,7 +2595,7 @@
         <v>gen[24]</v>
       </c>
       <c r="O35" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="T35" s="19"/>
       <c r="U35" s="19"/>
@@ -2784,7 +2785,7 @@
         <v>2</v>
       </c>
       <c r="O40" s="21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="41" spans="2:25" x14ac:dyDescent="0.3">
@@ -3117,7 +3118,7 @@
         <v>73</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F50" s="20" t="s">
         <v>92</v>
@@ -3125,7 +3126,7 @@
       <c r="G50" s="20"/>
       <c r="H50" s="20"/>
       <c r="I50" s="20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J50" s="20"/>
       <c r="K50" s="20"/>
@@ -3151,7 +3152,7 @@
         <v>74</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F51" s="20" t="s">
         <v>92</v>
@@ -3159,7 +3160,7 @@
       <c r="G51" s="20"/>
       <c r="H51" s="20"/>
       <c r="I51" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J51" s="20"/>
       <c r="K51" s="20"/>
@@ -3229,7 +3230,7 @@
       <c r="G53" s="20"/>
       <c r="H53" s="20"/>
       <c r="I53" s="20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J53" s="20"/>
       <c r="K53" s="20"/>
@@ -3241,7 +3242,7 @@
         <v>8~D</v>
       </c>
       <c r="N53" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O53" s="21"/>
     </row>
@@ -3295,13 +3296,13 @@
         <v>4</v>
       </c>
       <c r="G55" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="I55" s="20" t="s">
         <v>151</v>
-      </c>
-      <c r="H55" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="I55" s="20" t="s">
-        <v>152</v>
       </c>
       <c r="J55" s="20"/>
       <c r="K55" s="20"/>
@@ -3322,19 +3323,19 @@
         <v>79</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>92</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I56" s="20" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J56" s="20"/>
       <c r="K56" s="20"/>
@@ -3363,7 +3364,7 @@
         <v>7A</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>11</v>
@@ -3372,10 +3373,10 @@
         <v>92</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I57" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J57" s="20"/>
       <c r="K57" s="20"/>
@@ -3403,7 +3404,7 @@
         <v>7B</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>12</v>
@@ -3412,10 +3413,10 @@
         <v>92</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I58" s="20" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J58" s="20"/>
       <c r="K58" s="20"/>
@@ -3446,17 +3447,17 @@
         <v>7C</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F59" s="20" t="s">
         <v>92</v>
       </c>
       <c r="G59" s="20"/>
       <c r="H59" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="I59" s="20" t="s">
         <v>182</v>
-      </c>
-      <c r="I59" s="20" t="s">
-        <v>183</v>
       </c>
       <c r="J59" s="20"/>
       <c r="K59" s="20"/>
@@ -3485,19 +3486,19 @@
         <v>7D</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F60" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G60" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="G60" s="3" t="s">
+      <c r="H60" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="H60" s="3" t="s">
+      <c r="I60" s="20" t="s">
         <v>178</v>
-      </c>
-      <c r="I60" s="20" t="s">
-        <v>179</v>
       </c>
       <c r="J60" s="20"/>
       <c r="K60" s="20"/>
@@ -3531,21 +3532,21 @@
         <v>82</v>
       </c>
       <c r="F61" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="G61" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="G61" s="13" t="s">
-        <v>172</v>
-      </c>
       <c r="H61" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I61" s="20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J61" s="20"/>
       <c r="K61" s="20"/>
       <c r="L61" s="15" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M61" s="15"/>
       <c r="N61" s="15"/>
@@ -3556,32 +3557,32 @@
         <v>90</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7F</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F62" s="20" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G62" s="20"/>
       <c r="H62" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I62" s="20" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J62" s="20"/>
       <c r="K62" s="20"/>
       <c r="L62" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="M62" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N62" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L67,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L67,"-", -1))+1,"0"))</f>
@@ -3594,7 +3595,7 @@
         <v>90</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(D62) + 1),"~","FF")</f>
@@ -3609,7 +3610,7 @@
       <c r="G63" s="20"/>
       <c r="H63" s="20"/>
       <c r="I63" s="20" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J63" s="20"/>
       <c r="K63" s="20"/>
@@ -3618,7 +3619,7 @@
         <v>ex-2</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="N63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N62,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N62,"-", -1))+1,"0"))</f>
@@ -3628,19 +3629,19 @@
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B64" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="E64" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="C64" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="E64" s="3" t="s">
+      <c r="F64" s="3" t="s">
         <v>187</v>
-      </c>
-      <c r="F64" s="3" t="s">
-        <v>188</v>
       </c>
       <c r="G64" s="20"/>
       <c r="H64" s="20"/>
@@ -3652,7 +3653,7 @@
         <v>ex-3</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="N64" s="3" t="str">
         <f t="shared" ref="N64:N67" si="8">_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N63,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N63,"-", -1))+1,"0"))</f>
@@ -3663,16 +3664,16 @@
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B65" s="17"/>
       <c r="C65" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D65" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="E65" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="F65" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="F65" s="3" t="s">
-        <v>191</v>
       </c>
       <c r="G65" s="20"/>
       <c r="H65" s="20"/>
@@ -3684,7 +3685,7 @@
         <v>ex-4</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N65" s="3" t="str">
         <f t="shared" si="8"/>
@@ -3695,7 +3696,7 @@
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B66" s="17"/>
       <c r="C66" s="15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D66" s="20"/>
       <c r="E66" s="20"/>
@@ -3710,7 +3711,7 @@
         <v>ex-5</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="N66" s="3" t="str">
         <f t="shared" si="8"/>
@@ -3734,7 +3735,7 @@
         <v>ex-6</v>
       </c>
       <c r="M67" s="12" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="N67" s="12" t="str">
         <f t="shared" si="8"/>

</xml_diff>

<commit_message>
docs: ISA ABI section, cpu-test.dig paths, interrupt notes in todo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QJGhBeyFbVexj3aLG7xNkt
</commit_message>
<xml_diff>
--- a/document/ISA-32.xlsx
+++ b/document/ISA-32.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\digital computer 32\document\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\computer-32\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D6B8DB9-B1DF-459F-A3DF-A52E944852A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0220AE-48EB-45FD-B064-E477C4F7602A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7380" yWindow="675" windowWidth="28800" windowHeight="12915" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="211">
   <si>
     <t>opcode</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -389,10 +389,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PC = stack.pop(), end inter</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>user</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -481,10 +477,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>gen2[0~15]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Dumpling Industry's CPU-32 instruction set</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -665,10 +657,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ex-1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>istack</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -702,10 +690,6 @@
   </si>
   <si>
     <t>break</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>gen1[0~5]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -853,22 +837,10 @@
     <t>arg</t>
   </si>
   <si>
-    <t>at0</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>at1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>addr</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>kt</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>ABI/alias</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -878,6 +850,35 @@
   </si>
   <si>
     <t>arg,hret</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ex-0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>at</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>kt
+kt0,kt1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PC = istack.pop(), end inter</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gen[0~23]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>real id = register-id &lt;&lt; 3 | mode-id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ur/kn?</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1519,7 +1520,7 @@
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B6" s="22" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="23"/>
@@ -1581,7 +1582,7 @@
       <c r="J9" s="20"/>
       <c r="K9" s="20"/>
       <c r="L9" s="20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M9" s="20"/>
       <c r="N9" s="20"/>
@@ -1621,15 +1622,15 @@
         <v>39</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B11" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>45</v>
@@ -1647,7 +1648,7 @@
         <v>12</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I11" s="20" t="s">
         <v>55</v>
@@ -1655,7 +1656,7 @@
       <c r="J11" s="20"/>
       <c r="K11" s="20"/>
       <c r="L11" s="20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>26</v>
@@ -1665,12 +1666,12 @@
         <v>gen[0]</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B12" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C12" s="20"/>
       <c r="D12" s="3" t="str">
@@ -1687,7 +1688,7 @@
         <v>12</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I12" s="20" t="s">
         <v>56</v>
@@ -1704,12 +1705,12 @@
         <v>gen[1]</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B13" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C13" s="20"/>
       <c r="D13" s="3" t="str">
@@ -1741,12 +1742,12 @@
         <v>gen[2]</v>
       </c>
       <c r="O13" s="21" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C14" s="20"/>
       <c r="D14" s="3" t="str">
@@ -1763,7 +1764,7 @@
         <v>12</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I14" s="20" t="s">
         <v>58</v>
@@ -1783,7 +1784,7 @@
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="3" t="str">
@@ -1800,7 +1801,7 @@
         <v>12</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I15" s="20" t="s">
         <v>59</v>
@@ -1832,7 +1833,7 @@
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C16" s="20"/>
       <c r="D16" s="3" t="str">
@@ -1864,7 +1865,7 @@
         <v>gen[5]</v>
       </c>
       <c r="O16" s="21" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
@@ -1882,7 +1883,7 @@
     </row>
     <row r="17" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B17" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C17" s="20"/>
       <c r="D17" s="3" t="str">
@@ -1899,7 +1900,7 @@
         <v>12</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I17" s="20" t="s">
         <v>69</v>
@@ -1919,7 +1920,7 @@
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B18" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C18" s="20"/>
       <c r="D18" s="3" t="str">
@@ -1955,7 +1956,7 @@
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B19" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C19" s="20"/>
       <c r="D19" s="3" t="str">
@@ -1972,7 +1973,7 @@
         <v>12</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I19" s="20" t="s">
         <v>65</v>
@@ -1993,7 +1994,7 @@
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C20" s="20"/>
       <c r="D20" s="3" t="str">
@@ -2030,7 +2031,7 @@
     </row>
     <row r="21" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B21" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C21" s="20"/>
       <c r="D21" s="3" t="str">
@@ -2047,7 +2048,7 @@
         <v>12</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I21" s="20" t="s">
         <v>67</v>
@@ -2067,7 +2068,7 @@
     </row>
     <row r="22" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B22" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C22" s="20"/>
       <c r="D22" s="3" t="str">
@@ -2106,7 +2107,7 @@
     </row>
     <row r="23" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B23" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C23" s="20"/>
       <c r="D23" s="3" t="str">
@@ -2114,7 +2115,7 @@
         <v>0C</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>11</v>
@@ -2123,10 +2124,10 @@
         <v>12</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I23" s="20" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J23" s="20"/>
       <c r="K23" s="20"/>
@@ -2147,7 +2148,7 @@
     </row>
     <row r="24" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B24" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C24" s="20"/>
       <c r="D24" s="3" t="str">
@@ -2155,7 +2156,7 @@
         <v>0D</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>11</v>
@@ -2165,7 +2166,7 @@
       </c>
       <c r="H24" s="20"/>
       <c r="I24" s="20" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J24" s="20"/>
       <c r="K24" s="20"/>
@@ -2179,12 +2180,12 @@
         <v>gen[13]</v>
       </c>
       <c r="O24" s="21" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C25" s="20"/>
       <c r="D25" s="3" t="str">
@@ -2192,7 +2193,7 @@
         <v>0E</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>11</v>
@@ -2201,10 +2202,10 @@
         <v>12</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I25" s="20" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J25" s="20"/>
       <c r="K25" s="20"/>
@@ -2221,7 +2222,7 @@
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C26" s="20"/>
       <c r="D26" s="3" t="str">
@@ -2229,7 +2230,7 @@
         <v>0F</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>11</v>
@@ -2239,7 +2240,7 @@
       </c>
       <c r="H26" s="20"/>
       <c r="I26" s="20" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J26" s="20"/>
       <c r="K26" s="20"/>
@@ -2256,7 +2257,7 @@
     </row>
     <row r="27" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B27" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C27" s="20"/>
       <c r="D27" s="3" t="str">
@@ -2264,7 +2265,7 @@
         <v>10</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>11</v>
@@ -2273,7 +2274,7 @@
         <v>12</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I27" s="20" t="s">
         <v>61</v>
@@ -2293,7 +2294,7 @@
     </row>
     <row r="28" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B28" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C28" s="20"/>
       <c r="D28" s="3" t="str">
@@ -2301,7 +2302,7 @@
         <v>11</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>11</v>
@@ -2310,10 +2311,10 @@
         <v>12</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I28" s="20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="J28" s="20"/>
       <c r="K28" s="20"/>
@@ -2330,7 +2331,7 @@
     </row>
     <row r="29" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B29" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C29" s="20"/>
       <c r="D29" s="3" t="str">
@@ -2338,7 +2339,7 @@
         <v>12</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>11</v>
@@ -2365,7 +2366,7 @@
     </row>
     <row r="30" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B30" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C30" s="20"/>
       <c r="D30" s="3" t="str">
@@ -2373,7 +2374,7 @@
         <v>13</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>11</v>
@@ -2382,7 +2383,7 @@
         <v>12</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I30" s="20" t="s">
         <v>63</v>
@@ -2402,7 +2403,7 @@
     </row>
     <row r="31" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B31" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C31" s="20"/>
       <c r="D31" s="3" t="str">
@@ -2410,7 +2411,7 @@
         <v>14</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>11</v>
@@ -2419,10 +2420,10 @@
         <v>12</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I31" s="20" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="J31" s="20"/>
       <c r="K31" s="20"/>
@@ -2439,7 +2440,7 @@
     </row>
     <row r="32" spans="2:31" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C32" s="20"/>
       <c r="D32" s="3" t="str">
@@ -2447,7 +2448,7 @@
         <v>15</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>11</v>
@@ -2471,12 +2472,12 @@
         <v>gen[21]</v>
       </c>
       <c r="O32" s="8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B33" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C33" s="20"/>
       <c r="D33" s="3" t="str">
@@ -2484,19 +2485,19 @@
         <v>16</v>
       </c>
       <c r="E33" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G33" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="H33" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I33" s="20" t="s">
         <v>114</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="I33" s="20" t="s">
-        <v>116</v>
       </c>
       <c r="J33" s="20"/>
       <c r="K33" s="20"/>
@@ -2509,13 +2510,13 @@
         <f t="shared" si="3"/>
         <v>gen[22]</v>
       </c>
-      <c r="O33" s="8" t="s">
-        <v>205</v>
+      <c r="O33" s="16" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="34" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B34" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C34" s="20"/>
       <c r="D34" s="3" t="str">
@@ -2523,7 +2524,7 @@
         <v>17</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>12</v>
@@ -2533,7 +2534,7 @@
       </c>
       <c r="H34" s="20"/>
       <c r="I34" s="20" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="J34" s="20"/>
       <c r="K34" s="20"/>
@@ -2546,11 +2547,9 @@
         <f t="shared" si="3"/>
         <v>gen[23]</v>
       </c>
-      <c r="O34" s="8" t="s">
-        <v>207</v>
-      </c>
+      <c r="O34" s="21"/>
       <c r="R34" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="T34" s="19"/>
       <c r="U34" s="19"/>
@@ -2561,7 +2560,7 @@
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C35" s="20"/>
       <c r="D35" s="3" t="str">
@@ -2569,19 +2568,19 @@
         <v>18</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I35" s="20" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J35" s="20"/>
       <c r="K35" s="20"/>
@@ -2595,7 +2594,7 @@
         <v>gen[24]</v>
       </c>
       <c r="O35" s="8" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="T35" s="19"/>
       <c r="U35" s="19"/>
@@ -2606,7 +2605,7 @@
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C36" s="20"/>
       <c r="D36" s="3" t="str">
@@ -2614,7 +2613,7 @@
         <v>19</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>12</v>
@@ -2624,7 +2623,7 @@
       </c>
       <c r="H36" s="20"/>
       <c r="I36" s="20" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="J36" s="20"/>
       <c r="K36" s="20"/>
@@ -2634,15 +2633,15 @@
         <v>19</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="O36" s="8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B37" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C37" s="20" t="s">
         <v>47</v>
@@ -2667,7 +2666,7 @@
       <c r="J37" s="20"/>
       <c r="K37" s="20"/>
       <c r="L37" s="20" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M37" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2677,12 +2676,12 @@
         <v>6</v>
       </c>
       <c r="O37" s="21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="38" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B38" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C38" s="20"/>
       <c r="D38" s="3" t="str">
@@ -2690,7 +2689,7 @@
         <v>1B</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>11</v>
@@ -2700,7 +2699,7 @@
       </c>
       <c r="H38" s="20"/>
       <c r="I38" s="20" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J38" s="20"/>
       <c r="K38" s="20"/>
@@ -2716,7 +2715,7 @@
     </row>
     <row r="39" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B39" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C39" s="20"/>
       <c r="D39" s="3" t="str">
@@ -2733,7 +2732,7 @@
         <v>12</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I39" s="20" t="s">
         <v>53</v>
@@ -2752,7 +2751,7 @@
     </row>
     <row r="40" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B40" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>52</v>
@@ -2762,20 +2761,20 @@
         <v>1D</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F40" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G40" s="20"/>
       <c r="H40" s="20"/>
       <c r="I40" s="20" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J40" s="20"/>
       <c r="K40" s="20"/>
       <c r="L40" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M40" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2785,12 +2784,12 @@
         <v>2</v>
       </c>
       <c r="O40" s="21" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="41" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B41" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C41" s="20" t="s">
         <v>3</v>
@@ -2806,7 +2805,7 @@
         <v>11</v>
       </c>
       <c r="G41" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H41" s="20"/>
       <c r="I41" s="20" t="s">
@@ -2815,7 +2814,7 @@
       <c r="J41" s="20"/>
       <c r="K41" s="20"/>
       <c r="L41" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M41" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2829,7 +2828,7 @@
     </row>
     <row r="42" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B42" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C42" s="20"/>
       <c r="D42" s="3" t="str">
@@ -2843,7 +2842,7 @@
         <v>12</v>
       </c>
       <c r="G42" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H42" s="20"/>
       <c r="I42" s="20" t="s">
@@ -2852,7 +2851,7 @@
       <c r="J42" s="20"/>
       <c r="K42" s="20"/>
       <c r="L42" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M42" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2865,7 +2864,7 @@
     </row>
     <row r="43" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B43" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C43" s="20" t="s">
         <v>51</v>
@@ -2898,7 +2897,7 @@
     </row>
     <row r="44" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B44" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C44" s="20"/>
       <c r="D44" s="3" t="str">
@@ -2924,16 +2923,16 @@
         <v>46</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N44" s="20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O44" s="21"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B45" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C45" s="20" t="s">
         <v>52</v>
@@ -2958,7 +2957,7 @@
       <c r="J45" s="20"/>
       <c r="K45" s="20"/>
       <c r="L45" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M45" s="4" t="s">
         <v>26</v>
@@ -2970,7 +2969,7 @@
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B46" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C46" s="20"/>
       <c r="D46" s="3" t="str">
@@ -2978,7 +2977,7 @@
         <v>68~6F</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>4</v>
@@ -2993,7 +2992,7 @@
       <c r="J46" s="20"/>
       <c r="K46" s="20"/>
       <c r="L46" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M46" s="3" t="str">
         <f t="shared" ref="M46:M52" si="5">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M45)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M45)+1))</f>
@@ -3006,7 +3005,7 @@
     </row>
     <row r="47" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B47" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C47" s="20"/>
       <c r="D47" s="4" t="str">
@@ -3029,7 +3028,7 @@
       <c r="J47" s="20"/>
       <c r="K47" s="20"/>
       <c r="L47" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M47" s="3" t="str">
         <f t="shared" si="5"/>
@@ -3042,7 +3041,7 @@
     </row>
     <row r="48" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B48" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C48" s="20"/>
       <c r="D48" s="3" t="str">
@@ -3053,7 +3052,7 @@
         <v>49</v>
       </c>
       <c r="F48" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G48" s="20"/>
       <c r="H48" s="20"/>
@@ -3063,20 +3062,20 @@
       <c r="J48" s="20"/>
       <c r="K48" s="20"/>
       <c r="L48" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M48" s="3" t="str">
         <f t="shared" si="5"/>
         <v>03</v>
       </c>
       <c r="N48" s="20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O48" s="21"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C49" s="20"/>
       <c r="D49" s="3" t="str">
@@ -3087,7 +3086,7 @@
         <v>84</v>
       </c>
       <c r="F49" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G49" s="20"/>
       <c r="H49" s="20"/>
@@ -3097,20 +3096,20 @@
       <c r="J49" s="20"/>
       <c r="K49" s="20"/>
       <c r="L49" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M49" s="3" t="str">
         <f t="shared" si="5"/>
         <v>04</v>
       </c>
       <c r="N49" s="20" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O49" s="21"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C50" s="20"/>
       <c r="D50" s="3" t="str">
@@ -3118,33 +3117,33 @@
         <v>73</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="F50" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G50" s="20"/>
       <c r="H50" s="20"/>
       <c r="I50" s="20" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="J50" s="20"/>
       <c r="K50" s="20"/>
       <c r="L50" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M50" s="3" t="str">
         <f t="shared" si="5"/>
         <v>05</v>
       </c>
       <c r="N50" s="20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O50" s="21"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C51" s="20"/>
       <c r="D51" s="3" t="str">
@@ -3152,20 +3151,20 @@
         <v>74</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="F51" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G51" s="20"/>
       <c r="H51" s="20"/>
       <c r="I51" s="20" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="J51" s="20"/>
       <c r="K51" s="20"/>
       <c r="L51" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M51" s="3" t="str">
         <f t="shared" si="5"/>
@@ -3178,7 +3177,7 @@
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C52" s="20"/>
       <c r="D52" s="3" t="str">
@@ -3189,7 +3188,7 @@
         <v>37</v>
       </c>
       <c r="F52" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G52" s="20"/>
       <c r="H52" s="20"/>
@@ -3199,7 +3198,7 @@
       <c r="J52" s="20"/>
       <c r="K52" s="20"/>
       <c r="L52" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M52" s="3" t="str">
         <f t="shared" si="5"/>
@@ -3212,7 +3211,7 @@
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C53" s="20" t="s">
         <v>50</v>
@@ -3222,33 +3221,33 @@
         <v>76</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F53" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G53" s="20"/>
       <c r="H53" s="20"/>
       <c r="I53" s="20" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J53" s="20"/>
       <c r="K53" s="20"/>
       <c r="L53" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M53" s="3" t="str">
-        <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(M52) + 1),"~",DEC2HEX(HEX2DEC(M52) + 6))</f>
-        <v>8~D</v>
+        <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(M52) + 1),"~",DEC2HEX(HEX2DEC(M52) + 24))</f>
+        <v>8~1F</v>
       </c>
       <c r="N53" s="20" t="s">
-        <v>167</v>
+        <v>208</v>
       </c>
       <c r="O53" s="21"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C54" s="20"/>
       <c r="D54" s="3" t="str">
@@ -3259,30 +3258,25 @@
         <v>87</v>
       </c>
       <c r="F54" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G54" s="20"/>
       <c r="H54" s="20"/>
       <c r="I54" s="20" t="s">
-        <v>88</v>
+        <v>207</v>
       </c>
       <c r="J54" s="20"/>
       <c r="K54" s="20"/>
-      <c r="L54" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="M54" s="3" t="str">
-        <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(M53,LEN(M53)-FIND("~",M53,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(M53,LEN(M53)-FIND("~",M53,1))) + 16))</f>
-        <v>E~1D</v>
-      </c>
-      <c r="N54" s="20" t="s">
-        <v>111</v>
-      </c>
+      <c r="L54" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="M54" s="20"/>
+      <c r="N54" s="20"/>
       <c r="O54" s="21"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C55" s="20"/>
       <c r="D55" s="3" t="str">
@@ -3296,26 +3290,32 @@
         <v>4</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I55" s="20" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J55" s="20"/>
       <c r="K55" s="20"/>
-      <c r="L55" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="M55" s="20"/>
-      <c r="N55" s="20"/>
-      <c r="O55" s="21"/>
+      <c r="L55" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M55" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="N55" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O55" s="10" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C56" s="20"/>
       <c r="D56" s="3" t="str">
@@ -3323,38 +3323,39 @@
         <v>79</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I56" s="20" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="J56" s="20"/>
       <c r="K56" s="20"/>
-      <c r="L56" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="M56" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="N56" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="O56" s="10" t="s">
-        <v>91</v>
+      <c r="L56" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="M56" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N56" s="3" t="str">
+        <f>_xlfn.VALUETOTEXT(L59+1)</f>
+        <v>4</v>
+      </c>
+      <c r="O56" s="11" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C57" s="20" t="s">
         <v>47</v>
@@ -3364,39 +3365,40 @@
         <v>7A</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="I57" s="20" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="J57" s="20"/>
       <c r="K57" s="20"/>
-      <c r="L57" s="4" t="s">
+      <c r="L57" s="3" t="str">
+        <f>_xlfn.VALUETOTEXT(L56+1)</f>
+        <v>1</v>
+      </c>
+      <c r="M57" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="N57" s="3" t="str">
+        <f>_xlfn.VALUETOTEXT(N56+1)</f>
+        <v>5</v>
+      </c>
+      <c r="O57" s="11" t="s">
         <v>96</v>
-      </c>
-      <c r="M57" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="N57" s="3" t="str">
-        <f>_xlfn.VALUETOTEXT(L60+1)</f>
-        <v>4</v>
-      </c>
-      <c r="O57" s="11" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B58" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C58" s="20"/>
       <c r="D58" s="3" t="str">
@@ -3404,40 +3406,40 @@
         <v>7B</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="I58" s="20" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J58" s="20"/>
       <c r="K58" s="20"/>
       <c r="L58" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L57+1)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M58" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N58" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(N57+1)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O58" s="11" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C59" s="20" t="s">
         <v>38</v>
@@ -3447,30 +3449,30 @@
         <v>7C</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F59" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G59" s="20"/>
       <c r="H59" s="3" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="I59" s="20" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J59" s="20"/>
       <c r="K59" s="20"/>
       <c r="L59" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L58+1)</f>
-        <v>2</v>
-      </c>
-      <c r="M59" s="4" t="s">
-        <v>30</v>
+        <v>3</v>
+      </c>
+      <c r="M59" s="7" t="s">
+        <v>31</v>
       </c>
       <c r="N59" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(N58+1)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O59" s="11" t="s">
         <v>93</v>
@@ -3478,7 +3480,7 @@
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B60" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C60" s="20"/>
       <c r="D60" s="3" t="str">
@@ -3486,40 +3488,32 @@
         <v>7D</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="I60" s="20" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="J60" s="20"/>
       <c r="K60" s="20"/>
-      <c r="L60" s="3" t="str">
-        <f>_xlfn.VALUETOTEXT(L59+1)</f>
-        <v>3</v>
-      </c>
-      <c r="M60" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="N60" s="3" t="str">
-        <f>_xlfn.VALUETOTEXT(N59+1)</f>
-        <v>7</v>
-      </c>
-      <c r="O60" s="11" t="s">
-        <v>94</v>
-      </c>
+      <c r="L60" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="M60" s="20"/>
+      <c r="N60" s="20"/>
+      <c r="O60" s="21"/>
     </row>
     <row r="61" spans="2:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="9" t="s">
-        <v>90</v>
+        <v>210</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>82</v>
@@ -3532,21 +3526,21 @@
         <v>82</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="G61" s="13" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I61" s="20" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="J61" s="20"/>
       <c r="K61" s="20"/>
       <c r="L61" s="15" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="M61" s="15"/>
       <c r="N61" s="15"/>
@@ -3554,48 +3548,48 @@
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7F</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="F62" s="20" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="G62" s="20"/>
       <c r="H62" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="I62" s="20" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="J62" s="20"/>
       <c r="K62" s="20"/>
       <c r="L62" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="M62" s="3" t="s">
         <v>157</v>
-      </c>
-      <c r="M62" s="3" t="s">
-        <v>160</v>
       </c>
       <c r="N62" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L67,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L67,"-", -1))+1,"0"))</f>
-        <v>ex-7</v>
+        <v>ex-6</v>
       </c>
       <c r="O62" s="10"/>
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(D62) + 1),"~","FF")</f>
@@ -3605,43 +3599,43 @@
         <v>84</v>
       </c>
       <c r="F63" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G63" s="20"/>
       <c r="H63" s="20"/>
       <c r="I63" s="20" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="J63" s="20"/>
       <c r="K63" s="20"/>
       <c r="L63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L62,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L62,"-", -1))+1,"0"))</f>
-        <v>ex-2</v>
+        <v>ex-1</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="N63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N62,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N62,"-", -1))+1,"0"))</f>
-        <v>ex-8</v>
+        <v>ex-7</v>
       </c>
       <c r="O63" s="10"/>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B64" s="17" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="G64" s="20"/>
       <c r="H64" s="20"/>
@@ -3650,30 +3644,30 @@
       <c r="K64" s="20"/>
       <c r="L64" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L63,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L63,"-", -1))+1,"0"))</f>
-        <v>ex-3</v>
+        <v>ex-2</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="N64" s="3" t="str">
         <f t="shared" ref="N64:N67" si="8">_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N63,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N63,"-", -1))+1,"0"))</f>
-        <v>ex-9</v>
+        <v>ex-8</v>
       </c>
       <c r="O64" s="10"/>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B65" s="17"/>
       <c r="C65" s="3" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G65" s="20"/>
       <c r="H65" s="20"/>
@@ -3682,21 +3676,21 @@
       <c r="K65" s="20"/>
       <c r="L65" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L64,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L64,"-", -1))+1,"0"))</f>
-        <v>ex-4</v>
+        <v>ex-3</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N65" s="3" t="str">
         <f t="shared" si="8"/>
-        <v>ex-10</v>
+        <v>ex-9</v>
       </c>
       <c r="O65" s="10"/>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B66" s="17"/>
       <c r="C66" s="15" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D66" s="20"/>
       <c r="E66" s="20"/>
@@ -3708,14 +3702,14 @@
       <c r="K66" s="20"/>
       <c r="L66" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L65,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L65,"-", -1))+1,"0"))</f>
-        <v>ex-5</v>
+        <v>ex-4</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="N66" s="3" t="str">
         <f t="shared" si="8"/>
-        <v>ex-11</v>
+        <v>ex-10</v>
       </c>
       <c r="O66" s="10"/>
     </row>
@@ -3732,27 +3726,19 @@
       <c r="K67" s="31"/>
       <c r="L67" s="12" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L66,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L66,"-", -1))+1,"0"))</f>
-        <v>ex-6</v>
+        <v>ex-5</v>
       </c>
       <c r="M67" s="12" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="N67" s="12" t="str">
         <f t="shared" si="8"/>
-        <v>ex-12</v>
+        <v>ex-11</v>
       </c>
       <c r="O67" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="127">
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="N46:O46"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="N48:O48"/>
-    <mergeCell ref="N49:O49"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="I51:K51"/>
+  <mergeCells count="128">
     <mergeCell ref="C66:F67"/>
     <mergeCell ref="G64:K67"/>
     <mergeCell ref="I61:K61"/>
@@ -3763,26 +3749,21 @@
     <mergeCell ref="I63:K63"/>
     <mergeCell ref="N50:O50"/>
     <mergeCell ref="N53:O53"/>
-    <mergeCell ref="N54:O54"/>
     <mergeCell ref="I57:K57"/>
     <mergeCell ref="I59:K59"/>
     <mergeCell ref="I60:K60"/>
-    <mergeCell ref="L55:O55"/>
+    <mergeCell ref="L54:O54"/>
     <mergeCell ref="F54:H54"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="L60:O60"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="N46:O46"/>
+    <mergeCell ref="N47:O47"/>
+    <mergeCell ref="N48:O48"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="I51:K51"/>
     <mergeCell ref="F53:H53"/>
     <mergeCell ref="C53:C56"/>
     <mergeCell ref="C57:C58"/>
@@ -3802,9 +3783,11 @@
     <mergeCell ref="L9:O9"/>
     <mergeCell ref="O16:O23"/>
     <mergeCell ref="O24:O31"/>
-    <mergeCell ref="L11:L36"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="O13:O15"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G41:H41"/>
     <mergeCell ref="C45:C52"/>
     <mergeCell ref="I28:K28"/>
     <mergeCell ref="I32:K32"/>
@@ -3821,7 +3804,14 @@
     <mergeCell ref="F50:H50"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="F49:H49"/>
-    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="G38:H38"/>
     <mergeCell ref="T35:V35"/>
     <mergeCell ref="W35:Y35"/>
     <mergeCell ref="N44:O44"/>
@@ -3832,6 +3822,10 @@
     <mergeCell ref="I50:K50"/>
     <mergeCell ref="N45:O45"/>
     <mergeCell ref="O37:O39"/>
+    <mergeCell ref="L11:L36"/>
+    <mergeCell ref="O13:O15"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="O33:O34"/>
     <mergeCell ref="B9:K9"/>
     <mergeCell ref="I12:K12"/>
     <mergeCell ref="I30:K30"/>
@@ -3848,6 +3842,7 @@
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="I11:K11"/>
+    <mergeCell ref="C11:C36"/>
     <mergeCell ref="L61:O61"/>
     <mergeCell ref="B64:B67"/>
     <mergeCell ref="AF15:AG15"/>

</xml_diff>

<commit_message>
cpu[wip]: INT/MMU development (interst/interld, MMU-BL, store-buffer8-debug)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QJGhBeyFbVexj3aLG7xNkt
</commit_message>
<xml_diff>
--- a/document/ISA-32.xlsx
+++ b/document/ISA-32.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\computer-32\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0220AE-48EB-45FD-B064-E477C4F7602A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CBA0B7B-7CD7-4B81-8B47-199DED668AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="216">
   <si>
     <t>opcode</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -369,10 +369,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>intervec</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>nop</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -625,27 +621,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>interpri</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>m(0~255)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>int_vec[id] = base + imm</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>int_pri[id] = imm</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>d(0~63)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>m(0~15)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -874,11 +850,50 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>real id = register-id &lt;&lt; 3 | mode-id</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ur/kn?</t>
+    <t>interst</t>
+  </si>
+  <si>
+    <t>base</t>
+  </si>
+  <si>
+    <t>interld</t>
+  </si>
+  <si>
+    <t>dest</t>
+  </si>
+  <si>
+    <t>u.u</t>
+  </si>
+  <si>
+    <t>inter vec</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>intvec/pri[id] = base + imm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>md: b7, vec(0)/pri(1)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>id, b0-5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>real id = register-id&lt;&lt;3 | mode-id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>md | id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>md-id = md&lt;&lt;3 | id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dest = intvec/pri[id]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1076,7 +1091,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1125,19 +1140,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1170,8 +1176,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1519,78 +1540,78 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="24"/>
+      <c r="B6" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
+      <c r="O6" s="21"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="25"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="26"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="26"/>
-      <c r="N7" s="26"/>
-      <c r="O7" s="27"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="24"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="28"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="29"/>
-      <c r="L8" s="29"/>
-      <c r="M8" s="29"/>
-      <c r="N8" s="29"/>
-      <c r="O8" s="30"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
+      <c r="M8" s="26"/>
+      <c r="N8" s="26"/>
+      <c r="O8" s="27"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
-      <c r="J9" s="20"/>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="M9" s="20"/>
-      <c r="N9" s="20"/>
-      <c r="O9" s="21"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="18"/>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>46</v>
@@ -1610,11 +1631,11 @@
       <c r="H10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="20" t="s">
+      <c r="I10" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
       <c r="L10" s="3" t="s">
         <v>46</v>
       </c>
@@ -1622,17 +1643,17 @@
         <v>39</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B11" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>45</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -1648,15 +1669,15 @@
         <v>12</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I11" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20" t="s">
-        <v>100</v>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>26</v>
@@ -1666,14 +1687,14 @@
         <v>gen[0]</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B12" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C12" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C12" s="16"/>
       <c r="D12" s="3" t="str">
         <f t="shared" ref="D12:D36" si="1">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D11)+1))</f>
         <v>01</v>
@@ -1688,14 +1709,14 @@
         <v>12</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I12" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I12" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
       <c r="M12" s="3" t="str">
         <f t="shared" ref="M12:M42" si="2">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M11)+1))</f>
         <v>01</v>
@@ -1705,14 +1726,14 @@
         <v>gen[1]</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B13" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C13" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C13" s="16"/>
       <c r="D13" s="3" t="str">
         <f t="shared" si="1"/>
         <v>02</v>
@@ -1723,16 +1744,16 @@
       <c r="F13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20" t="s">
+      <c r="H13" s="16"/>
+      <c r="I13" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J13" s="20"/>
-      <c r="K13" s="20"/>
-      <c r="L13" s="20"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
       <c r="M13" s="3" t="str">
         <f t="shared" si="2"/>
         <v>02</v>
@@ -1741,15 +1762,15 @@
         <f t="shared" si="0"/>
         <v>gen[2]</v>
       </c>
-      <c r="O13" s="21" t="s">
-        <v>199</v>
+      <c r="O13" s="18" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C14" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C14" s="16"/>
       <c r="D14" s="3" t="str">
         <f t="shared" si="1"/>
         <v>03</v>
@@ -1764,14 +1785,14 @@
         <v>12</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I14" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I14" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
-      <c r="L14" s="20"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
       <c r="M14" s="3" t="str">
         <f t="shared" si="2"/>
         <v>03</v>
@@ -1780,13 +1801,13 @@
         <f t="shared" si="0"/>
         <v>gen[3]</v>
       </c>
-      <c r="O14" s="21"/>
+      <c r="O14" s="18"/>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C15" s="16"/>
       <c r="D15" s="3" t="str">
         <f t="shared" si="1"/>
         <v>04</v>
@@ -1801,14 +1822,14 @@
         <v>12</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I15" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I15" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="J15" s="20"/>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
       <c r="M15" s="3" t="str">
         <f t="shared" si="2"/>
         <v>04</v>
@@ -1817,25 +1838,25 @@
         <f t="shared" si="0"/>
         <v>gen[4]</v>
       </c>
-      <c r="O15" s="21"/>
-      <c r="U15" s="19"/>
-      <c r="V15" s="19"/>
-      <c r="W15" s="19"/>
-      <c r="X15" s="19"/>
-      <c r="Y15" s="19"/>
-      <c r="Z15" s="19"/>
-      <c r="AA15" s="19"/>
-      <c r="AB15" s="19"/>
-      <c r="AC15" s="19"/>
-      <c r="AD15" s="19"/>
-      <c r="AF15" s="19"/>
-      <c r="AG15" s="19"/>
+      <c r="O15" s="18"/>
+      <c r="U15" s="28"/>
+      <c r="V15" s="28"/>
+      <c r="W15" s="28"/>
+      <c r="X15" s="28"/>
+      <c r="Y15" s="28"/>
+      <c r="Z15" s="28"/>
+      <c r="AA15" s="28"/>
+      <c r="AB15" s="28"/>
+      <c r="AC15" s="28"/>
+      <c r="AD15" s="28"/>
+      <c r="AF15" s="28"/>
+      <c r="AG15" s="28"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C16" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C16" s="16"/>
       <c r="D16" s="3" t="str">
         <f t="shared" si="1"/>
         <v>05</v>
@@ -1846,16 +1867,16 @@
       <c r="F16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20" t="s">
+      <c r="H16" s="16"/>
+      <c r="I16" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
       <c r="M16" s="3" t="str">
         <f t="shared" si="2"/>
         <v>05</v>
@@ -1864,8 +1885,8 @@
         <f t="shared" si="0"/>
         <v>gen[5]</v>
       </c>
-      <c r="O16" s="21" t="s">
-        <v>145</v>
+      <c r="O16" s="18" t="s">
+        <v>144</v>
       </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
@@ -1883,9 +1904,9 @@
     </row>
     <row r="17" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B17" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C17" s="16"/>
       <c r="D17" s="3" t="str">
         <f t="shared" si="1"/>
         <v>06</v>
@@ -1900,14 +1921,14 @@
         <v>12</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I17" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I17" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20"/>
-      <c r="L17" s="20"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
       <c r="M17" s="3" t="str">
         <f t="shared" si="2"/>
         <v>06</v>
@@ -1916,13 +1937,13 @@
         <f t="shared" ref="N17:N35" si="3">_xlfn.TEXTJOIN(,TRUE,"gen[",_xlfn.VALUETOTEXT(HEX2DEC(M17)),"]")</f>
         <v>gen[6]</v>
       </c>
-      <c r="O17" s="21"/>
+      <c r="O17" s="18"/>
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B18" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C18" s="16"/>
       <c r="D18" s="3" t="str">
         <f t="shared" si="1"/>
         <v>07</v>
@@ -1933,16 +1954,16 @@
       <c r="F18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20" t="s">
+      <c r="H18" s="16"/>
+      <c r="I18" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
       <c r="M18" s="3" t="str">
         <f t="shared" si="2"/>
         <v>07</v>
@@ -1951,14 +1972,14 @@
         <f t="shared" si="3"/>
         <v>gen[7]</v>
       </c>
-      <c r="O18" s="21"/>
+      <c r="O18" s="18"/>
       <c r="AE18" s="2"/>
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B19" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C19" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C19" s="16"/>
       <c r="D19" s="3" t="str">
         <f t="shared" si="1"/>
         <v>08</v>
@@ -1973,14 +1994,14 @@
         <v>12</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I19" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I19" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
       <c r="M19" s="3" t="str">
         <f t="shared" si="2"/>
         <v>08</v>
@@ -1989,14 +2010,14 @@
         <f t="shared" si="3"/>
         <v>gen[8]</v>
       </c>
-      <c r="O19" s="21"/>
+      <c r="O19" s="18"/>
       <c r="V19" s="2"/>
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C20" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C20" s="16"/>
       <c r="D20" s="3" t="str">
         <f t="shared" si="1"/>
         <v>09</v>
@@ -2007,16 +2028,16 @@
       <c r="F20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20" t="s">
+      <c r="H20" s="16"/>
+      <c r="I20" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20"/>
-      <c r="L20" s="20"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
       <c r="M20" s="3" t="str">
         <f t="shared" si="2"/>
         <v>09</v>
@@ -2025,15 +2046,15 @@
         <f t="shared" si="3"/>
         <v>gen[9]</v>
       </c>
-      <c r="O20" s="21"/>
+      <c r="O20" s="18"/>
       <c r="R20" s="2"/>
       <c r="V20" s="2"/>
     </row>
     <row r="21" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B21" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C21" s="16"/>
       <c r="D21" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0A</v>
@@ -2048,14 +2069,14 @@
         <v>12</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I21" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I21" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
-      <c r="L21" s="20"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
       <c r="M21" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0A</v>
@@ -2064,13 +2085,13 @@
         <f t="shared" si="3"/>
         <v>gen[10]</v>
       </c>
-      <c r="O21" s="21"/>
+      <c r="O21" s="18"/>
     </row>
     <row r="22" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B22" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C22" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C22" s="16"/>
       <c r="D22" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0B</v>
@@ -2081,16 +2102,16 @@
       <c r="F22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="G22" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H22" s="20"/>
-      <c r="I22" s="20" t="s">
+      <c r="H22" s="16"/>
+      <c r="I22" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="J22" s="20"/>
-      <c r="K22" s="20"/>
-      <c r="L22" s="20"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
       <c r="M22" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0B</v>
@@ -2099,7 +2120,7 @@
         <f t="shared" si="3"/>
         <v>gen[11]</v>
       </c>
-      <c r="O22" s="21"/>
+      <c r="O22" s="18"/>
       <c r="S22" s="1"/>
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
@@ -2107,15 +2128,15 @@
     </row>
     <row r="23" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B23" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C23" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C23" s="16"/>
       <c r="D23" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0C</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>11</v>
@@ -2124,14 +2145,14 @@
         <v>12</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I23" s="20" t="s">
-        <v>125</v>
-      </c>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
-      <c r="L23" s="20"/>
+        <v>90</v>
+      </c>
+      <c r="I23" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
       <c r="M23" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0C</v>
@@ -2140,7 +2161,7 @@
         <f t="shared" si="3"/>
         <v>gen[12]</v>
       </c>
-      <c r="O23" s="21"/>
+      <c r="O23" s="18"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
@@ -2148,29 +2169,29 @@
     </row>
     <row r="24" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B24" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C24" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C24" s="16"/>
       <c r="D24" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0D</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H24" s="20"/>
-      <c r="I24" s="20" t="s">
-        <v>133</v>
-      </c>
-      <c r="J24" s="20"/>
-      <c r="K24" s="20"/>
-      <c r="L24" s="20"/>
+      <c r="H24" s="16"/>
+      <c r="I24" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="16"/>
       <c r="M24" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0D</v>
@@ -2179,21 +2200,21 @@
         <f t="shared" si="3"/>
         <v>gen[13]</v>
       </c>
-      <c r="O24" s="21" t="s">
-        <v>146</v>
+      <c r="O24" s="18" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C25" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C25" s="16"/>
       <c r="D25" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0E</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>11</v>
@@ -2202,14 +2223,14 @@
         <v>12</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I25" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="J25" s="20"/>
-      <c r="K25" s="20"/>
-      <c r="L25" s="20"/>
+        <v>90</v>
+      </c>
+      <c r="I25" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="J25" s="16"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
       <c r="M25" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0E</v>
@@ -2218,33 +2239,33 @@
         <f t="shared" si="3"/>
         <v>gen[14]</v>
       </c>
-      <c r="O25" s="21"/>
+      <c r="O25" s="18"/>
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C26" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C26" s="16"/>
       <c r="D26" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0F</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G26" s="20" t="s">
+      <c r="G26" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="20"/>
-      <c r="I26" s="20" t="s">
-        <v>132</v>
-      </c>
-      <c r="J26" s="20"/>
-      <c r="K26" s="20"/>
-      <c r="L26" s="20"/>
+      <c r="H26" s="16"/>
+      <c r="I26" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="J26" s="16"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
       <c r="M26" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0F</v>
@@ -2253,19 +2274,19 @@
         <f t="shared" si="3"/>
         <v>gen[15]</v>
       </c>
-      <c r="O26" s="21"/>
+      <c r="O26" s="18"/>
     </row>
     <row r="27" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B27" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C27" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C27" s="16"/>
       <c r="D27" s="3" t="str">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>11</v>
@@ -2274,14 +2295,14 @@
         <v>12</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I27" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I27" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="J27" s="20"/>
-      <c r="K27" s="20"/>
-      <c r="L27" s="20"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="16"/>
       <c r="M27" s="3" t="str">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -2290,19 +2311,19 @@
         <f t="shared" si="3"/>
         <v>gen[16]</v>
       </c>
-      <c r="O27" s="21"/>
+      <c r="O27" s="18"/>
     </row>
     <row r="28" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B28" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C28" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C28" s="16"/>
       <c r="D28" s="3" t="str">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>11</v>
@@ -2311,14 +2332,14 @@
         <v>12</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I28" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20"/>
-      <c r="L28" s="20"/>
+        <v>90</v>
+      </c>
+      <c r="I28" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
       <c r="M28" s="3" t="str">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -2327,33 +2348,33 @@
         <f t="shared" si="3"/>
         <v>gen[17]</v>
       </c>
-      <c r="O28" s="21"/>
+      <c r="O28" s="18"/>
     </row>
     <row r="29" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B29" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C29" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C29" s="16"/>
       <c r="D29" s="3" t="str">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="G29" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H29" s="20"/>
-      <c r="I29" s="20" t="s">
+      <c r="H29" s="16"/>
+      <c r="I29" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J29" s="20"/>
-      <c r="K29" s="20"/>
-      <c r="L29" s="20"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
       <c r="M29" s="3" t="str">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -2362,19 +2383,19 @@
         <f t="shared" si="3"/>
         <v>gen[18]</v>
       </c>
-      <c r="O29" s="21"/>
+      <c r="O29" s="18"/>
     </row>
     <row r="30" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B30" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C30" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C30" s="16"/>
       <c r="D30" s="3" t="str">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>11</v>
@@ -2383,14 +2404,14 @@
         <v>12</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I30" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I30" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
-      <c r="L30" s="20"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
       <c r="M30" s="3" t="str">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -2399,19 +2420,19 @@
         <f t="shared" si="3"/>
         <v>gen[19]</v>
       </c>
-      <c r="O30" s="21"/>
+      <c r="O30" s="18"/>
     </row>
     <row r="31" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B31" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C31" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C31" s="16"/>
       <c r="D31" s="3" t="str">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>11</v>
@@ -2420,14 +2441,14 @@
         <v>12</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I31" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
-      <c r="L31" s="20"/>
+        <v>90</v>
+      </c>
+      <c r="I31" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="16"/>
       <c r="M31" s="3" t="str">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -2436,33 +2457,33 @@
         <f t="shared" si="3"/>
         <v>gen[20]</v>
       </c>
-      <c r="O31" s="21"/>
+      <c r="O31" s="18"/>
     </row>
     <row r="32" spans="2:31" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C32" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C32" s="16"/>
       <c r="D32" s="3" t="str">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="G32" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H32" s="20"/>
-      <c r="I32" s="20" t="s">
+      <c r="H32" s="16"/>
+      <c r="I32" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="J32" s="20"/>
-      <c r="K32" s="20"/>
-      <c r="L32" s="20"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
+      <c r="L32" s="16"/>
       <c r="M32" s="3" t="str">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -2472,36 +2493,36 @@
         <v>gen[21]</v>
       </c>
       <c r="O32" s="8" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B33" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C33" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C33" s="16"/>
       <c r="D33" s="3" t="str">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="E33" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="G33" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="H33" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I33" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="H33" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I33" s="20" t="s">
-        <v>114</v>
-      </c>
-      <c r="J33" s="20"/>
-      <c r="K33" s="20"/>
-      <c r="L33" s="20"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="16"/>
+      <c r="L33" s="16"/>
       <c r="M33" s="3" t="str">
         <f t="shared" si="2"/>
         <v>16</v>
@@ -2510,35 +2531,35 @@
         <f t="shared" si="3"/>
         <v>gen[22]</v>
       </c>
-      <c r="O33" s="16" t="s">
-        <v>206</v>
+      <c r="O33" s="29" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B34" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C34" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C34" s="16"/>
       <c r="D34" s="3" t="str">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="20" t="s">
+      <c r="G34" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H34" s="20"/>
-      <c r="I34" s="20" t="s">
-        <v>140</v>
-      </c>
-      <c r="J34" s="20"/>
-      <c r="K34" s="20"/>
-      <c r="L34" s="20"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="J34" s="16"/>
+      <c r="K34" s="16"/>
+      <c r="L34" s="16"/>
       <c r="M34" s="3" t="str">
         <f t="shared" si="2"/>
         <v>17</v>
@@ -2547,44 +2568,44 @@
         <f t="shared" si="3"/>
         <v>gen[23]</v>
       </c>
-      <c r="O34" s="21"/>
+      <c r="O34" s="18"/>
       <c r="R34" t="s">
-        <v>134</v>
-      </c>
-      <c r="T34" s="19"/>
-      <c r="U34" s="19"/>
-      <c r="V34" s="19"/>
-      <c r="W34" s="19"/>
-      <c r="X34" s="19"/>
-      <c r="Y34" s="19"/>
+        <v>133</v>
+      </c>
+      <c r="T34" s="28"/>
+      <c r="U34" s="28"/>
+      <c r="V34" s="28"/>
+      <c r="W34" s="28"/>
+      <c r="X34" s="28"/>
+      <c r="Y34" s="28"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C35" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C35" s="16"/>
       <c r="D35" s="3" t="str">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="E35" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I35" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="F35" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I35" s="20" t="s">
-        <v>127</v>
-      </c>
-      <c r="J35" s="20"/>
-      <c r="K35" s="20"/>
-      <c r="L35" s="20"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16"/>
       <c r="M35" s="3" t="str">
         <f t="shared" si="2"/>
         <v>18</v>
@@ -2594,56 +2615,56 @@
         <v>gen[24]</v>
       </c>
       <c r="O35" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="T35" s="19"/>
-      <c r="U35" s="19"/>
-      <c r="V35" s="19"/>
-      <c r="W35" s="19"/>
-      <c r="X35" s="19"/>
-      <c r="Y35" s="19"/>
+        <v>194</v>
+      </c>
+      <c r="T35" s="28"/>
+      <c r="U35" s="28"/>
+      <c r="V35" s="28"/>
+      <c r="W35" s="28"/>
+      <c r="X35" s="28"/>
+      <c r="Y35" s="28"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C36" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C36" s="16"/>
       <c r="D36" s="3" t="str">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="20" t="s">
+      <c r="G36" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H36" s="20"/>
-      <c r="I36" s="20" t="s">
-        <v>139</v>
-      </c>
-      <c r="J36" s="20"/>
-      <c r="K36" s="20"/>
-      <c r="L36" s="20"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="J36" s="16"/>
+      <c r="K36" s="16"/>
+      <c r="L36" s="16"/>
       <c r="M36" s="3" t="str">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O36" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B37" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C37" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C37" s="16" t="s">
         <v>47</v>
       </c>
       <c r="D37" s="3" t="str">
@@ -2656,17 +2677,17 @@
       <c r="F37" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G37" s="20" t="s">
+      <c r="G37" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H37" s="20"/>
-      <c r="I37" s="20" t="s">
+      <c r="H37" s="16"/>
+      <c r="I37" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="J37" s="20"/>
-      <c r="K37" s="20"/>
-      <c r="L37" s="20" t="s">
-        <v>101</v>
+      <c r="J37" s="16"/>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16" t="s">
+        <v>100</v>
       </c>
       <c r="M37" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2675,35 +2696,35 @@
       <c r="N37" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="O37" s="21" t="s">
-        <v>107</v>
+      <c r="O37" s="18" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="38" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B38" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C38" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C38" s="16"/>
       <c r="D38" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1B</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G38" s="20" t="s">
+      <c r="G38" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H38" s="20"/>
-      <c r="I38" s="20" t="s">
-        <v>138</v>
-      </c>
-      <c r="J38" s="20"/>
-      <c r="K38" s="20"/>
-      <c r="L38" s="20"/>
+      <c r="H38" s="16"/>
+      <c r="I38" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="J38" s="16"/>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16"/>
       <c r="M38" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1B</v>
@@ -2711,13 +2732,13 @@
       <c r="N38" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="21"/>
+      <c r="O38" s="18"/>
     </row>
     <row r="39" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B39" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C39" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C39" s="16"/>
       <c r="D39" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1C</v>
@@ -2732,14 +2753,14 @@
         <v>12</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I39" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I39" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="J39" s="20"/>
-      <c r="K39" s="20"/>
-      <c r="L39" s="20"/>
+      <c r="J39" s="16"/>
+      <c r="K39" s="16"/>
+      <c r="L39" s="16"/>
       <c r="M39" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1C</v>
@@ -2747,11 +2768,11 @@
       <c r="N39" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O39" s="21"/>
+      <c r="O39" s="18"/>
     </row>
     <row r="40" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B40" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>52</v>
@@ -2761,20 +2782,20 @@
         <v>1D</v>
       </c>
       <c r="E40" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F40" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="F40" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20" t="s">
-        <v>144</v>
-      </c>
-      <c r="J40" s="20"/>
-      <c r="K40" s="20"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="16"/>
       <c r="L40" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M40" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2783,15 +2804,15 @@
       <c r="N40" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O40" s="21" t="s">
-        <v>158</v>
+      <c r="O40" s="18" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="41" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B41" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C41" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D41" s="3" t="str">
@@ -2804,17 +2825,17 @@
       <c r="F41" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G41" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="H41" s="20"/>
-      <c r="I41" s="20" t="s">
+      <c r="G41" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="H41" s="16"/>
+      <c r="I41" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="J41" s="20"/>
-      <c r="K41" s="20"/>
+      <c r="J41" s="16"/>
+      <c r="K41" s="16"/>
       <c r="L41" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M41" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2823,14 +2844,14 @@
       <c r="N41" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="O41" s="21"/>
+      <c r="O41" s="18"/>
       <c r="T41" s="2"/>
     </row>
     <row r="42" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B42" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C42" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C42" s="16"/>
       <c r="D42" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1F</v>
@@ -2841,17 +2862,17 @@
       <c r="F42" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G42" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="H42" s="20"/>
-      <c r="I42" s="20" t="s">
+      <c r="G42" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="H42" s="16"/>
+      <c r="I42" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="J42" s="20"/>
-      <c r="K42" s="20"/>
+      <c r="J42" s="16"/>
+      <c r="K42" s="16"/>
       <c r="L42" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M42" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2860,13 +2881,13 @@
       <c r="N42" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="O42" s="21"/>
+      <c r="O42" s="18"/>
     </row>
     <row r="43" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B43" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C43" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C43" s="16" t="s">
         <v>51</v>
       </c>
       <c r="D43" s="3" t="str">
@@ -2879,27 +2900,27 @@
       <c r="F43" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G43" s="20" t="s">
+      <c r="G43" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H43" s="20"/>
-      <c r="I43" s="20" t="s">
+      <c r="H43" s="16"/>
+      <c r="I43" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="J43" s="20"/>
-      <c r="K43" s="20"/>
-      <c r="L43" s="20" t="s">
+      <c r="J43" s="16"/>
+      <c r="K43" s="16"/>
+      <c r="L43" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="M43" s="20"/>
-      <c r="N43" s="20"/>
-      <c r="O43" s="21"/>
+      <c r="M43" s="16"/>
+      <c r="N43" s="16"/>
+      <c r="O43" s="18"/>
     </row>
     <row r="44" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B44" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C44" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C44" s="16"/>
       <c r="D44" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 32))</f>
         <v>40~5F</v>
@@ -2910,31 +2931,31 @@
       <c r="F44" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G44" s="20" t="s">
+      <c r="G44" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H44" s="20"/>
-      <c r="I44" s="20" t="s">
+      <c r="H44" s="16"/>
+      <c r="I44" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="J44" s="20"/>
-      <c r="K44" s="20"/>
+      <c r="J44" s="16"/>
+      <c r="K44" s="16"/>
       <c r="L44" s="6" t="s">
         <v>46</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="N44" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="O44" s="21"/>
+        <v>107</v>
+      </c>
+      <c r="N44" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="O44" s="18"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B45" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C45" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>52</v>
       </c>
       <c r="D45" s="3" t="str">
@@ -2947,67 +2968,67 @@
       <c r="F45" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G45" s="20" t="s">
+      <c r="G45" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H45" s="20"/>
-      <c r="I45" s="20" t="s">
+      <c r="H45" s="16"/>
+      <c r="I45" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="J45" s="20"/>
-      <c r="K45" s="20"/>
+      <c r="J45" s="16"/>
+      <c r="K45" s="16"/>
       <c r="L45" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M45" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="N45" s="20" t="s">
+      <c r="N45" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="O45" s="21"/>
+      <c r="O45" s="18"/>
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B46" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C46" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C46" s="16"/>
       <c r="D46" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 8))</f>
         <v>68~6F</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G46" s="20" t="s">
+      <c r="G46" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H46" s="20"/>
-      <c r="I46" s="20" t="s">
+      <c r="H46" s="16"/>
+      <c r="I46" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="J46" s="20"/>
-      <c r="K46" s="20"/>
+      <c r="J46" s="16"/>
+      <c r="K46" s="16"/>
       <c r="L46" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M46" s="3" t="str">
         <f t="shared" ref="M46:M52" si="5">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M45)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M45)+1))</f>
         <v>01</v>
       </c>
-      <c r="N46" s="20" t="s">
+      <c r="N46" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="O46" s="21"/>
+      <c r="O46" s="18"/>
     </row>
     <row r="47" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B47" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C47" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C47" s="16"/>
       <c r="D47" s="4" t="str">
         <f>DEC2HEX(HEX2DEC(RIGHT(D46,LEN(D46)-FIND("~",D46,1))) + 1)</f>
         <v>70</v>
@@ -3018,32 +3039,32 @@
       <c r="F47" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G47" s="20" t="s">
+      <c r="G47" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H47" s="20"/>
-      <c r="I47" s="20" t="s">
+      <c r="H47" s="16"/>
+      <c r="I47" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="J47" s="20"/>
-      <c r="K47" s="20"/>
+      <c r="J47" s="16"/>
+      <c r="K47" s="16"/>
       <c r="L47" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M47" s="3" t="str">
         <f t="shared" si="5"/>
         <v>02</v>
       </c>
-      <c r="N47" s="20" t="s">
+      <c r="N47" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="O47" s="21"/>
+      <c r="O47" s="18"/>
     </row>
     <row r="48" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B48" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C48" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C48" s="16"/>
       <c r="D48" s="3" t="str">
         <f t="shared" ref="D48:D54" si="6">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D47)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D47)+1))</f>
         <v>71</v>
@@ -3051,135 +3072,135 @@
       <c r="E48" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F48" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G48" s="20"/>
-      <c r="H48" s="20"/>
-      <c r="I48" s="20" t="s">
+      <c r="F48" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G48" s="16"/>
+      <c r="H48" s="16"/>
+      <c r="I48" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="J48" s="20"/>
-      <c r="K48" s="20"/>
+      <c r="J48" s="16"/>
+      <c r="K48" s="16"/>
       <c r="L48" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M48" s="3" t="str">
         <f t="shared" si="5"/>
         <v>03</v>
       </c>
-      <c r="N48" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="O48" s="21"/>
+      <c r="N48" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="O48" s="18"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C49" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C49" s="16"/>
       <c r="D49" s="3" t="str">
         <f t="shared" si="6"/>
         <v>72</v>
       </c>
       <c r="E49" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F49" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G49" s="16"/>
+      <c r="H49" s="16"/>
+      <c r="I49" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="F49" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G49" s="20"/>
-      <c r="H49" s="20"/>
-      <c r="I49" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="J49" s="20"/>
-      <c r="K49" s="20"/>
+      <c r="J49" s="16"/>
+      <c r="K49" s="16"/>
       <c r="L49" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M49" s="3" t="str">
         <f t="shared" si="5"/>
         <v>04</v>
       </c>
-      <c r="N49" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="O49" s="21"/>
+      <c r="N49" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="O49" s="18"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C50" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C50" s="16"/>
       <c r="D50" s="3" t="str">
         <f t="shared" si="6"/>
         <v>73</v>
       </c>
       <c r="E50" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F50" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G50" s="16"/>
+      <c r="H50" s="16"/>
+      <c r="I50" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="F50" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G50" s="20"/>
-      <c r="H50" s="20"/>
-      <c r="I50" s="20" t="s">
-        <v>169</v>
-      </c>
-      <c r="J50" s="20"/>
-      <c r="K50" s="20"/>
+      <c r="J50" s="16"/>
+      <c r="K50" s="16"/>
       <c r="L50" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M50" s="3" t="str">
         <f t="shared" si="5"/>
         <v>05</v>
       </c>
-      <c r="N50" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="O50" s="21"/>
+      <c r="N50" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="O50" s="18"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C51" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C51" s="16"/>
       <c r="D51" s="3" t="str">
         <f t="shared" si="6"/>
         <v>74</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="F51" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="J51" s="20"/>
-      <c r="K51" s="20"/>
+        <v>156</v>
+      </c>
+      <c r="F51" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G51" s="16"/>
+      <c r="H51" s="16"/>
+      <c r="I51" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="J51" s="16"/>
+      <c r="K51" s="16"/>
       <c r="L51" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M51" s="3" t="str">
         <f t="shared" si="5"/>
         <v>06</v>
       </c>
-      <c r="N51" s="20" t="s">
+      <c r="N51" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="O51" s="21"/>
+      <c r="O51" s="18"/>
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C52" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C52" s="16"/>
       <c r="D52" s="3" t="str">
         <f t="shared" si="6"/>
         <v>75</v>
@@ -3187,33 +3208,33 @@
       <c r="E52" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F52" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="20" t="s">
+      <c r="F52" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G52" s="16"/>
+      <c r="H52" s="16"/>
+      <c r="I52" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="J52" s="20"/>
-      <c r="K52" s="20"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="16"/>
       <c r="L52" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M52" s="3" t="str">
         <f t="shared" si="5"/>
         <v>07</v>
       </c>
-      <c r="N52" s="20" t="s">
+      <c r="N52" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="O52" s="21"/>
+      <c r="O52" s="18"/>
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C53" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C53" s="16" t="s">
         <v>50</v>
       </c>
       <c r="D53" s="3" t="str">
@@ -3221,126 +3242,126 @@
         <v>76</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="F53" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G53" s="20"/>
-      <c r="H53" s="20"/>
-      <c r="I53" s="20" t="s">
-        <v>170</v>
-      </c>
-      <c r="J53" s="20"/>
-      <c r="K53" s="20"/>
+        <v>97</v>
+      </c>
+      <c r="F53" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G53" s="16"/>
+      <c r="H53" s="16"/>
+      <c r="I53" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="J53" s="16"/>
+      <c r="K53" s="16"/>
       <c r="L53" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M53" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(M52) + 1),"~",DEC2HEX(HEX2DEC(M52) + 24))</f>
         <v>8~1F</v>
       </c>
-      <c r="N53" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="O53" s="21"/>
+      <c r="N53" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="O53" s="18"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C54" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C54" s="16"/>
       <c r="D54" s="3" t="str">
         <f t="shared" si="6"/>
         <v>77</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="F54" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="20" t="s">
-        <v>207</v>
-      </c>
-      <c r="J54" s="20"/>
-      <c r="K54" s="20"/>
-      <c r="L54" s="20" t="s">
-        <v>109</v>
-      </c>
-      <c r="M54" s="20"/>
-      <c r="N54" s="20"/>
-      <c r="O54" s="21"/>
+        <v>86</v>
+      </c>
+      <c r="F54" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G54" s="16"/>
+      <c r="H54" s="16"/>
+      <c r="I54" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="J54" s="16"/>
+      <c r="K54" s="16"/>
+      <c r="L54" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="M54" s="16"/>
+      <c r="N54" s="16"/>
+      <c r="O54" s="18"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C55" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C55" s="16"/>
       <c r="D55" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D54)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D54)+1))</f>
         <v>78</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>83</v>
+        <v>203</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>4</v>
+        <v>204</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I55" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="J55" s="20"/>
-      <c r="K55" s="20"/>
+        <v>213</v>
+      </c>
+      <c r="I55" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="J55" s="16"/>
+      <c r="K55" s="16"/>
       <c r="L55" s="5" t="s">
         <v>39</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N55" s="5" t="s">
         <v>39</v>
       </c>
       <c r="O55" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C56" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C56" s="16"/>
       <c r="D56" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D55)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D55)+1))</f>
         <v>79</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>147</v>
+        <v>205</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>91</v>
+        <v>206</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>152</v>
+        <v>207</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I56" s="20" t="s">
-        <v>150</v>
-      </c>
-      <c r="J56" s="20"/>
-      <c r="K56" s="20"/>
+        <v>213</v>
+      </c>
+      <c r="I56" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="J56" s="16"/>
+      <c r="K56" s="16"/>
       <c r="L56" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M56" s="7" t="s">
         <v>27</v>
@@ -3350,14 +3371,14 @@
         <v>4</v>
       </c>
       <c r="O56" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C57" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="C57" s="16" t="s">
         <v>47</v>
       </c>
       <c r="D57" s="3" t="str">
@@ -3365,22 +3386,22 @@
         <v>7A</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="I57" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="J57" s="20"/>
-      <c r="K57" s="20"/>
+        <v>182</v>
+      </c>
+      <c r="I57" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="J57" s="16"/>
+      <c r="K57" s="16"/>
       <c r="L57" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L56+1)</f>
         <v>1</v>
@@ -3393,35 +3414,35 @@
         <v>5</v>
       </c>
       <c r="O57" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B58" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C58" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C58" s="16"/>
       <c r="D58" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D57)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D57)+1))</f>
         <v>7B</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="I58" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="J58" s="20"/>
-      <c r="K58" s="20"/>
+        <v>182</v>
+      </c>
+      <c r="I58" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="J58" s="16"/>
+      <c r="K58" s="16"/>
       <c r="L58" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L57+1)</f>
         <v>2</v>
@@ -3434,14 +3455,14 @@
         <v>6</v>
       </c>
       <c r="O58" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C59" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="C59" s="16" t="s">
         <v>38</v>
       </c>
       <c r="D59" s="3" t="str">
@@ -3449,20 +3470,20 @@
         <v>7C</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="F59" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G59" s="20"/>
+        <v>170</v>
+      </c>
+      <c r="F59" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G59" s="16"/>
       <c r="H59" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="I59" s="20" t="s">
-        <v>178</v>
-      </c>
-      <c r="J59" s="20"/>
-      <c r="K59" s="20"/>
+        <v>171</v>
+      </c>
+      <c r="I59" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="J59" s="16"/>
+      <c r="K59" s="16"/>
       <c r="L59" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L58+1)</f>
         <v>3</v>
@@ -3475,45 +3496,45 @@
         <v>7</v>
       </c>
       <c r="O59" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B60" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C60" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C60" s="16"/>
       <c r="D60" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7D</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="I60" s="20" t="s">
-        <v>174</v>
-      </c>
-      <c r="J60" s="20"/>
-      <c r="K60" s="20"/>
-      <c r="L60" s="20" t="s">
-        <v>209</v>
-      </c>
-      <c r="M60" s="20"/>
-      <c r="N60" s="20"/>
-      <c r="O60" s="21"/>
+        <v>167</v>
+      </c>
+      <c r="I60" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="J60" s="16"/>
+      <c r="K60" s="16"/>
+      <c r="L60" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="M60" s="16"/>
+      <c r="N60" s="16"/>
+      <c r="O60" s="18"/>
     </row>
     <row r="61" spans="2:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="9" t="s">
-        <v>210</v>
+        <v>88</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>82</v>
@@ -3526,57 +3547,57 @@
         <v>82</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G61" s="13" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="I61" s="20" t="s">
-        <v>191</v>
-      </c>
-      <c r="J61" s="20"/>
-      <c r="K61" s="20"/>
+        <v>159</v>
+      </c>
+      <c r="I61" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="J61" s="16"/>
+      <c r="K61" s="16"/>
       <c r="L61" s="15" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="M61" s="15"/>
       <c r="N61" s="15"/>
-      <c r="O61" s="16"/>
+      <c r="O61" s="29"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7F</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="F62" s="20" t="s">
-        <v>194</v>
-      </c>
-      <c r="G62" s="20"/>
+        <v>186</v>
+      </c>
+      <c r="F62" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="G62" s="16"/>
       <c r="H62" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="I62" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="J62" s="20"/>
-      <c r="K62" s="20"/>
+        <v>187</v>
+      </c>
+      <c r="I62" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="J62" s="16"/>
+      <c r="K62" s="16"/>
       <c r="L62" s="4" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="M62" s="3" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="N62" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L67,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L67,"-", -1))+1,"0"))</f>
@@ -3586,34 +3607,34 @@
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(D62) + 1),"~","FF")</f>
         <v>80~FF</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="F63" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G63" s="20"/>
-      <c r="H63" s="20"/>
-      <c r="I63" s="20" t="s">
-        <v>180</v>
-      </c>
-      <c r="J63" s="20"/>
-      <c r="K63" s="20"/>
+        <v>83</v>
+      </c>
+      <c r="F63" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G63" s="16"/>
+      <c r="H63" s="16"/>
+      <c r="I63" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="J63" s="16"/>
+      <c r="K63" s="16"/>
       <c r="L63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L62,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L62,"-", -1))+1,"0"))</f>
         <v>ex-1</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="N63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N62,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N62,"-", -1))+1,"0"))</f>
@@ -3622,32 +3643,34 @@
       <c r="O63" s="10"/>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B64" s="17" t="s">
-        <v>181</v>
+      <c r="B64" s="30" t="s">
+        <v>175</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="G64" s="20"/>
-      <c r="H64" s="20"/>
-      <c r="I64" s="20"/>
-      <c r="J64" s="20"/>
-      <c r="K64" s="20"/>
+        <v>177</v>
+      </c>
+      <c r="G64" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="H64" s="16"/>
+      <c r="I64" s="32"/>
+      <c r="J64" s="32"/>
+      <c r="K64" s="32"/>
       <c r="L64" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L63,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L63,"-", -1))+1,"0"))</f>
         <v>ex-2</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="N64" s="3" t="str">
         <f t="shared" ref="N64:N67" si="8">_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N63,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N63,"-", -1))+1,"0"))</f>
@@ -3656,30 +3679,32 @@
       <c r="O64" s="10"/>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B65" s="17"/>
+      <c r="B65" s="30"/>
       <c r="C65" s="3" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="G65" s="20"/>
-      <c r="H65" s="20"/>
-      <c r="I65" s="20"/>
-      <c r="J65" s="20"/>
-      <c r="K65" s="20"/>
+        <v>180</v>
+      </c>
+      <c r="G65" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="H65" s="16"/>
+      <c r="I65" s="32"/>
+      <c r="J65" s="32"/>
+      <c r="K65" s="32"/>
       <c r="L65" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L64,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L64,"-", -1))+1,"0"))</f>
         <v>ex-3</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="N65" s="3" t="str">
         <f t="shared" si="8"/>
@@ -3688,24 +3713,26 @@
       <c r="O65" s="10"/>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B66" s="17"/>
+      <c r="B66" s="30"/>
       <c r="C66" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="D66" s="20"/>
-      <c r="E66" s="20"/>
-      <c r="F66" s="20"/>
-      <c r="G66" s="20"/>
-      <c r="H66" s="20"/>
-      <c r="I66" s="20"/>
-      <c r="J66" s="20"/>
-      <c r="K66" s="20"/>
+        <v>191</v>
+      </c>
+      <c r="D66" s="16"/>
+      <c r="E66" s="16"/>
+      <c r="F66" s="16"/>
+      <c r="G66" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="H66" s="16"/>
+      <c r="I66" s="32"/>
+      <c r="J66" s="32"/>
+      <c r="K66" s="32"/>
       <c r="L66" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L65,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L65,"-", -1))+1,"0"))</f>
         <v>ex-4</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="N66" s="3" t="str">
         <f t="shared" si="8"/>
@@ -3714,22 +3741,24 @@
       <c r="O66" s="10"/>
     </row>
     <row r="67" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B67" s="18"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="31"/>
-      <c r="E67" s="31"/>
-      <c r="F67" s="31"/>
-      <c r="G67" s="31"/>
-      <c r="H67" s="31"/>
-      <c r="I67" s="31"/>
-      <c r="J67" s="31"/>
-      <c r="K67" s="31"/>
+      <c r="B67" s="31"/>
+      <c r="C67" s="17"/>
+      <c r="D67" s="17"/>
+      <c r="E67" s="17"/>
+      <c r="F67" s="17"/>
+      <c r="G67" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="H67" s="17"/>
+      <c r="I67" s="33"/>
+      <c r="J67" s="33"/>
+      <c r="K67" s="33"/>
       <c r="L67" s="12" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L66,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L66,"-", -1))+1,"0"))</f>
         <v>ex-5</v>
       </c>
       <c r="M67" s="12" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="N67" s="12" t="str">
         <f t="shared" si="8"/>
@@ -3738,30 +3767,91 @@
       <c r="O67" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="128">
-    <mergeCell ref="C66:F67"/>
-    <mergeCell ref="G64:K67"/>
-    <mergeCell ref="I61:K61"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="O40:O42"/>
-    <mergeCell ref="F63:H63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="N53:O53"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="L54:O54"/>
-    <mergeCell ref="F54:H54"/>
-    <mergeCell ref="L60:O60"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="N46:O46"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="N48:O48"/>
-    <mergeCell ref="N49:O49"/>
+  <mergeCells count="131">
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="L61:O61"/>
+    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="AF15:AG15"/>
+    <mergeCell ref="L43:O43"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="I49:K49"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="U15:AB15"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="C11:C36"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="N44:O44"/>
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:K46"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="O37:O39"/>
+    <mergeCell ref="L11:L36"/>
+    <mergeCell ref="O13:O15"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="O33:O34"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="C45:C52"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="F51:H51"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="C43:C44"/>
     <mergeCell ref="C37:C39"/>
     <mergeCell ref="I51:K51"/>
     <mergeCell ref="F53:H53"/>
@@ -3786,87 +3876,29 @@
     <mergeCell ref="I54:K54"/>
     <mergeCell ref="I58:K58"/>
     <mergeCell ref="C41:C42"/>
+    <mergeCell ref="C66:F67"/>
+    <mergeCell ref="I61:K61"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="O40:O42"/>
+    <mergeCell ref="F63:H63"/>
+    <mergeCell ref="I63:K63"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="N53:O53"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="I59:K59"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="L54:O54"/>
+    <mergeCell ref="F54:H54"/>
+    <mergeCell ref="L60:O60"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="N46:O46"/>
+    <mergeCell ref="N47:O47"/>
+    <mergeCell ref="N48:O48"/>
+    <mergeCell ref="N49:O49"/>
     <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="C45:C52"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="N44:O44"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="O37:O39"/>
-    <mergeCell ref="L11:L36"/>
-    <mergeCell ref="O13:O15"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="O33:O34"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="L61:O61"/>
-    <mergeCell ref="B64:B67"/>
-    <mergeCell ref="AF15:AG15"/>
-    <mergeCell ref="L43:O43"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="T34:V34"/>
-    <mergeCell ref="W34:Y34"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="U15:AB15"/>
-    <mergeCell ref="I55:K55"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
docs: update ISA-32.xlsx (interst/interld sheet)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QJGhBeyFbVexj3aLG7xNkt
</commit_message>
<xml_diff>
--- a/document/ISA-32.xlsx
+++ b/document/ISA-32.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\computer-32\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0220AE-48EB-45FD-B064-E477C4F7602A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CBA0B7B-7CD7-4B81-8B47-199DED668AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="216">
   <si>
     <t>opcode</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -369,10 +369,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>intervec</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>nop</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -625,27 +621,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>interpri</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>m(0~255)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>int_vec[id] = base + imm</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>int_pri[id] = imm</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>d(0~63)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>m(0~15)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -874,11 +850,50 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>real id = register-id &lt;&lt; 3 | mode-id</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ur/kn?</t>
+    <t>interst</t>
+  </si>
+  <si>
+    <t>base</t>
+  </si>
+  <si>
+    <t>interld</t>
+  </si>
+  <si>
+    <t>dest</t>
+  </si>
+  <si>
+    <t>u.u</t>
+  </si>
+  <si>
+    <t>inter vec</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>intvec/pri[id] = base + imm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>md: b7, vec(0)/pri(1)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>id, b0-5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>real id = register-id&lt;&lt;3 | mode-id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>md | id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>md-id = md&lt;&lt;3 | id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dest = intvec/pri[id]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1076,7 +1091,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1125,19 +1140,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1170,8 +1176,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1519,78 +1540,78 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="24"/>
+      <c r="B6" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
+      <c r="O6" s="21"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="25"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="26"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="26"/>
-      <c r="N7" s="26"/>
-      <c r="O7" s="27"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="24"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="28"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="29"/>
-      <c r="L8" s="29"/>
-      <c r="M8" s="29"/>
-      <c r="N8" s="29"/>
-      <c r="O8" s="30"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
+      <c r="M8" s="26"/>
+      <c r="N8" s="26"/>
+      <c r="O8" s="27"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
-      <c r="J9" s="20"/>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="M9" s="20"/>
-      <c r="N9" s="20"/>
-      <c r="O9" s="21"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="18"/>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>46</v>
@@ -1610,11 +1631,11 @@
       <c r="H10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="20" t="s">
+      <c r="I10" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
       <c r="L10" s="3" t="s">
         <v>46</v>
       </c>
@@ -1622,17 +1643,17 @@
         <v>39</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B11" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>45</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -1648,15 +1669,15 @@
         <v>12</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I11" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20" t="s">
-        <v>100</v>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16" t="s">
+        <v>99</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>26</v>
@@ -1666,14 +1687,14 @@
         <v>gen[0]</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B12" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C12" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C12" s="16"/>
       <c r="D12" s="3" t="str">
         <f t="shared" ref="D12:D36" si="1">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D11)+1))</f>
         <v>01</v>
@@ -1688,14 +1709,14 @@
         <v>12</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I12" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I12" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
       <c r="M12" s="3" t="str">
         <f t="shared" ref="M12:M42" si="2">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M11)+1))</f>
         <v>01</v>
@@ -1705,14 +1726,14 @@
         <v>gen[1]</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B13" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C13" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C13" s="16"/>
       <c r="D13" s="3" t="str">
         <f t="shared" si="1"/>
         <v>02</v>
@@ -1723,16 +1744,16 @@
       <c r="F13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20" t="s">
+      <c r="H13" s="16"/>
+      <c r="I13" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="J13" s="20"/>
-      <c r="K13" s="20"/>
-      <c r="L13" s="20"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
       <c r="M13" s="3" t="str">
         <f t="shared" si="2"/>
         <v>02</v>
@@ -1741,15 +1762,15 @@
         <f t="shared" si="0"/>
         <v>gen[2]</v>
       </c>
-      <c r="O13" s="21" t="s">
-        <v>199</v>
+      <c r="O13" s="18" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C14" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C14" s="16"/>
       <c r="D14" s="3" t="str">
         <f t="shared" si="1"/>
         <v>03</v>
@@ -1764,14 +1785,14 @@
         <v>12</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I14" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I14" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
-      <c r="L14" s="20"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
       <c r="M14" s="3" t="str">
         <f t="shared" si="2"/>
         <v>03</v>
@@ -1780,13 +1801,13 @@
         <f t="shared" si="0"/>
         <v>gen[3]</v>
       </c>
-      <c r="O14" s="21"/>
+      <c r="O14" s="18"/>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C15" s="16"/>
       <c r="D15" s="3" t="str">
         <f t="shared" si="1"/>
         <v>04</v>
@@ -1801,14 +1822,14 @@
         <v>12</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I15" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I15" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="J15" s="20"/>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
       <c r="M15" s="3" t="str">
         <f t="shared" si="2"/>
         <v>04</v>
@@ -1817,25 +1838,25 @@
         <f t="shared" si="0"/>
         <v>gen[4]</v>
       </c>
-      <c r="O15" s="21"/>
-      <c r="U15" s="19"/>
-      <c r="V15" s="19"/>
-      <c r="W15" s="19"/>
-      <c r="X15" s="19"/>
-      <c r="Y15" s="19"/>
-      <c r="Z15" s="19"/>
-      <c r="AA15" s="19"/>
-      <c r="AB15" s="19"/>
-      <c r="AC15" s="19"/>
-      <c r="AD15" s="19"/>
-      <c r="AF15" s="19"/>
-      <c r="AG15" s="19"/>
+      <c r="O15" s="18"/>
+      <c r="U15" s="28"/>
+      <c r="V15" s="28"/>
+      <c r="W15" s="28"/>
+      <c r="X15" s="28"/>
+      <c r="Y15" s="28"/>
+      <c r="Z15" s="28"/>
+      <c r="AA15" s="28"/>
+      <c r="AB15" s="28"/>
+      <c r="AC15" s="28"/>
+      <c r="AD15" s="28"/>
+      <c r="AF15" s="28"/>
+      <c r="AG15" s="28"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C16" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C16" s="16"/>
       <c r="D16" s="3" t="str">
         <f t="shared" si="1"/>
         <v>05</v>
@@ -1846,16 +1867,16 @@
       <c r="F16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20" t="s">
+      <c r="H16" s="16"/>
+      <c r="I16" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
       <c r="M16" s="3" t="str">
         <f t="shared" si="2"/>
         <v>05</v>
@@ -1864,8 +1885,8 @@
         <f t="shared" si="0"/>
         <v>gen[5]</v>
       </c>
-      <c r="O16" s="21" t="s">
-        <v>145</v>
+      <c r="O16" s="18" t="s">
+        <v>144</v>
       </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
@@ -1883,9 +1904,9 @@
     </row>
     <row r="17" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B17" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C17" s="16"/>
       <c r="D17" s="3" t="str">
         <f t="shared" si="1"/>
         <v>06</v>
@@ -1900,14 +1921,14 @@
         <v>12</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I17" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I17" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20"/>
-      <c r="L17" s="20"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
       <c r="M17" s="3" t="str">
         <f t="shared" si="2"/>
         <v>06</v>
@@ -1916,13 +1937,13 @@
         <f t="shared" ref="N17:N35" si="3">_xlfn.TEXTJOIN(,TRUE,"gen[",_xlfn.VALUETOTEXT(HEX2DEC(M17)),"]")</f>
         <v>gen[6]</v>
       </c>
-      <c r="O17" s="21"/>
+      <c r="O17" s="18"/>
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B18" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C18" s="16"/>
       <c r="D18" s="3" t="str">
         <f t="shared" si="1"/>
         <v>07</v>
@@ -1933,16 +1954,16 @@
       <c r="F18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20" t="s">
+      <c r="H18" s="16"/>
+      <c r="I18" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
       <c r="M18" s="3" t="str">
         <f t="shared" si="2"/>
         <v>07</v>
@@ -1951,14 +1972,14 @@
         <f t="shared" si="3"/>
         <v>gen[7]</v>
       </c>
-      <c r="O18" s="21"/>
+      <c r="O18" s="18"/>
       <c r="AE18" s="2"/>
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B19" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C19" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C19" s="16"/>
       <c r="D19" s="3" t="str">
         <f t="shared" si="1"/>
         <v>08</v>
@@ -1973,14 +1994,14 @@
         <v>12</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I19" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I19" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
       <c r="M19" s="3" t="str">
         <f t="shared" si="2"/>
         <v>08</v>
@@ -1989,14 +2010,14 @@
         <f t="shared" si="3"/>
         <v>gen[8]</v>
       </c>
-      <c r="O19" s="21"/>
+      <c r="O19" s="18"/>
       <c r="V19" s="2"/>
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C20" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C20" s="16"/>
       <c r="D20" s="3" t="str">
         <f t="shared" si="1"/>
         <v>09</v>
@@ -2007,16 +2028,16 @@
       <c r="F20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20" t="s">
+      <c r="H20" s="16"/>
+      <c r="I20" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20"/>
-      <c r="L20" s="20"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
       <c r="M20" s="3" t="str">
         <f t="shared" si="2"/>
         <v>09</v>
@@ -2025,15 +2046,15 @@
         <f t="shared" si="3"/>
         <v>gen[9]</v>
       </c>
-      <c r="O20" s="21"/>
+      <c r="O20" s="18"/>
       <c r="R20" s="2"/>
       <c r="V20" s="2"/>
     </row>
     <row r="21" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B21" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C21" s="16"/>
       <c r="D21" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0A</v>
@@ -2048,14 +2069,14 @@
         <v>12</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I21" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I21" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
-      <c r="L21" s="20"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
       <c r="M21" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0A</v>
@@ -2064,13 +2085,13 @@
         <f t="shared" si="3"/>
         <v>gen[10]</v>
       </c>
-      <c r="O21" s="21"/>
+      <c r="O21" s="18"/>
     </row>
     <row r="22" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B22" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C22" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C22" s="16"/>
       <c r="D22" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0B</v>
@@ -2081,16 +2102,16 @@
       <c r="F22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="G22" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H22" s="20"/>
-      <c r="I22" s="20" t="s">
+      <c r="H22" s="16"/>
+      <c r="I22" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="J22" s="20"/>
-      <c r="K22" s="20"/>
-      <c r="L22" s="20"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
       <c r="M22" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0B</v>
@@ -2099,7 +2120,7 @@
         <f t="shared" si="3"/>
         <v>gen[11]</v>
       </c>
-      <c r="O22" s="21"/>
+      <c r="O22" s="18"/>
       <c r="S22" s="1"/>
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
@@ -2107,15 +2128,15 @@
     </row>
     <row r="23" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B23" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C23" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C23" s="16"/>
       <c r="D23" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0C</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>11</v>
@@ -2124,14 +2145,14 @@
         <v>12</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I23" s="20" t="s">
-        <v>125</v>
-      </c>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
-      <c r="L23" s="20"/>
+        <v>90</v>
+      </c>
+      <c r="I23" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
       <c r="M23" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0C</v>
@@ -2140,7 +2161,7 @@
         <f t="shared" si="3"/>
         <v>gen[12]</v>
       </c>
-      <c r="O23" s="21"/>
+      <c r="O23" s="18"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
@@ -2148,29 +2169,29 @@
     </row>
     <row r="24" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B24" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C24" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C24" s="16"/>
       <c r="D24" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0D</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H24" s="20"/>
-      <c r="I24" s="20" t="s">
-        <v>133</v>
-      </c>
-      <c r="J24" s="20"/>
-      <c r="K24" s="20"/>
-      <c r="L24" s="20"/>
+      <c r="H24" s="16"/>
+      <c r="I24" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="16"/>
       <c r="M24" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0D</v>
@@ -2179,21 +2200,21 @@
         <f t="shared" si="3"/>
         <v>gen[13]</v>
       </c>
-      <c r="O24" s="21" t="s">
-        <v>146</v>
+      <c r="O24" s="18" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C25" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C25" s="16"/>
       <c r="D25" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0E</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>11</v>
@@ -2202,14 +2223,14 @@
         <v>12</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I25" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="J25" s="20"/>
-      <c r="K25" s="20"/>
-      <c r="L25" s="20"/>
+        <v>90</v>
+      </c>
+      <c r="I25" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="J25" s="16"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
       <c r="M25" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0E</v>
@@ -2218,33 +2239,33 @@
         <f t="shared" si="3"/>
         <v>gen[14]</v>
       </c>
-      <c r="O25" s="21"/>
+      <c r="O25" s="18"/>
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C26" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C26" s="16"/>
       <c r="D26" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0F</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G26" s="20" t="s">
+      <c r="G26" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="20"/>
-      <c r="I26" s="20" t="s">
-        <v>132</v>
-      </c>
-      <c r="J26" s="20"/>
-      <c r="K26" s="20"/>
-      <c r="L26" s="20"/>
+      <c r="H26" s="16"/>
+      <c r="I26" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="J26" s="16"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
       <c r="M26" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0F</v>
@@ -2253,19 +2274,19 @@
         <f t="shared" si="3"/>
         <v>gen[15]</v>
       </c>
-      <c r="O26" s="21"/>
+      <c r="O26" s="18"/>
     </row>
     <row r="27" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B27" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C27" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C27" s="16"/>
       <c r="D27" s="3" t="str">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>11</v>
@@ -2274,14 +2295,14 @@
         <v>12</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I27" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I27" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="J27" s="20"/>
-      <c r="K27" s="20"/>
-      <c r="L27" s="20"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="16"/>
       <c r="M27" s="3" t="str">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -2290,19 +2311,19 @@
         <f t="shared" si="3"/>
         <v>gen[16]</v>
       </c>
-      <c r="O27" s="21"/>
+      <c r="O27" s="18"/>
     </row>
     <row r="28" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B28" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C28" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C28" s="16"/>
       <c r="D28" s="3" t="str">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>11</v>
@@ -2311,14 +2332,14 @@
         <v>12</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I28" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20"/>
-      <c r="L28" s="20"/>
+        <v>90</v>
+      </c>
+      <c r="I28" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
       <c r="M28" s="3" t="str">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -2327,33 +2348,33 @@
         <f t="shared" si="3"/>
         <v>gen[17]</v>
       </c>
-      <c r="O28" s="21"/>
+      <c r="O28" s="18"/>
     </row>
     <row r="29" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B29" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C29" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C29" s="16"/>
       <c r="D29" s="3" t="str">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="G29" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H29" s="20"/>
-      <c r="I29" s="20" t="s">
+      <c r="H29" s="16"/>
+      <c r="I29" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="J29" s="20"/>
-      <c r="K29" s="20"/>
-      <c r="L29" s="20"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
       <c r="M29" s="3" t="str">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -2362,19 +2383,19 @@
         <f t="shared" si="3"/>
         <v>gen[18]</v>
       </c>
-      <c r="O29" s="21"/>
+      <c r="O29" s="18"/>
     </row>
     <row r="30" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B30" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C30" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C30" s="16"/>
       <c r="D30" s="3" t="str">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>11</v>
@@ -2383,14 +2404,14 @@
         <v>12</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I30" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I30" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
-      <c r="L30" s="20"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
       <c r="M30" s="3" t="str">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -2399,19 +2420,19 @@
         <f t="shared" si="3"/>
         <v>gen[19]</v>
       </c>
-      <c r="O30" s="21"/>
+      <c r="O30" s="18"/>
     </row>
     <row r="31" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B31" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C31" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C31" s="16"/>
       <c r="D31" s="3" t="str">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>11</v>
@@ -2420,14 +2441,14 @@
         <v>12</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I31" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
-      <c r="L31" s="20"/>
+        <v>90</v>
+      </c>
+      <c r="I31" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="16"/>
       <c r="M31" s="3" t="str">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -2436,33 +2457,33 @@
         <f t="shared" si="3"/>
         <v>gen[20]</v>
       </c>
-      <c r="O31" s="21"/>
+      <c r="O31" s="18"/>
     </row>
     <row r="32" spans="2:31" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C32" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C32" s="16"/>
       <c r="D32" s="3" t="str">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="G32" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H32" s="20"/>
-      <c r="I32" s="20" t="s">
+      <c r="H32" s="16"/>
+      <c r="I32" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="J32" s="20"/>
-      <c r="K32" s="20"/>
-      <c r="L32" s="20"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
+      <c r="L32" s="16"/>
       <c r="M32" s="3" t="str">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -2472,36 +2493,36 @@
         <v>gen[21]</v>
       </c>
       <c r="O32" s="8" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B33" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C33" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C33" s="16"/>
       <c r="D33" s="3" t="str">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="E33" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="G33" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="H33" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I33" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="H33" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I33" s="20" t="s">
-        <v>114</v>
-      </c>
-      <c r="J33" s="20"/>
-      <c r="K33" s="20"/>
-      <c r="L33" s="20"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="16"/>
+      <c r="L33" s="16"/>
       <c r="M33" s="3" t="str">
         <f t="shared" si="2"/>
         <v>16</v>
@@ -2510,35 +2531,35 @@
         <f t="shared" si="3"/>
         <v>gen[22]</v>
       </c>
-      <c r="O33" s="16" t="s">
-        <v>206</v>
+      <c r="O33" s="29" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B34" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C34" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C34" s="16"/>
       <c r="D34" s="3" t="str">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="20" t="s">
+      <c r="G34" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H34" s="20"/>
-      <c r="I34" s="20" t="s">
-        <v>140</v>
-      </c>
-      <c r="J34" s="20"/>
-      <c r="K34" s="20"/>
-      <c r="L34" s="20"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="J34" s="16"/>
+      <c r="K34" s="16"/>
+      <c r="L34" s="16"/>
       <c r="M34" s="3" t="str">
         <f t="shared" si="2"/>
         <v>17</v>
@@ -2547,44 +2568,44 @@
         <f t="shared" si="3"/>
         <v>gen[23]</v>
       </c>
-      <c r="O34" s="21"/>
+      <c r="O34" s="18"/>
       <c r="R34" t="s">
-        <v>134</v>
-      </c>
-      <c r="T34" s="19"/>
-      <c r="U34" s="19"/>
-      <c r="V34" s="19"/>
-      <c r="W34" s="19"/>
-      <c r="X34" s="19"/>
-      <c r="Y34" s="19"/>
+        <v>133</v>
+      </c>
+      <c r="T34" s="28"/>
+      <c r="U34" s="28"/>
+      <c r="V34" s="28"/>
+      <c r="W34" s="28"/>
+      <c r="X34" s="28"/>
+      <c r="Y34" s="28"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C35" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C35" s="16"/>
       <c r="D35" s="3" t="str">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="E35" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I35" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="F35" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I35" s="20" t="s">
-        <v>127</v>
-      </c>
-      <c r="J35" s="20"/>
-      <c r="K35" s="20"/>
-      <c r="L35" s="20"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16"/>
       <c r="M35" s="3" t="str">
         <f t="shared" si="2"/>
         <v>18</v>
@@ -2594,56 +2615,56 @@
         <v>gen[24]</v>
       </c>
       <c r="O35" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="T35" s="19"/>
-      <c r="U35" s="19"/>
-      <c r="V35" s="19"/>
-      <c r="W35" s="19"/>
-      <c r="X35" s="19"/>
-      <c r="Y35" s="19"/>
+        <v>194</v>
+      </c>
+      <c r="T35" s="28"/>
+      <c r="U35" s="28"/>
+      <c r="V35" s="28"/>
+      <c r="W35" s="28"/>
+      <c r="X35" s="28"/>
+      <c r="Y35" s="28"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C36" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C36" s="16"/>
       <c r="D36" s="3" t="str">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="20" t="s">
+      <c r="G36" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H36" s="20"/>
-      <c r="I36" s="20" t="s">
-        <v>139</v>
-      </c>
-      <c r="J36" s="20"/>
-      <c r="K36" s="20"/>
-      <c r="L36" s="20"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="J36" s="16"/>
+      <c r="K36" s="16"/>
+      <c r="L36" s="16"/>
       <c r="M36" s="3" t="str">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O36" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B37" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C37" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C37" s="16" t="s">
         <v>47</v>
       </c>
       <c r="D37" s="3" t="str">
@@ -2656,17 +2677,17 @@
       <c r="F37" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G37" s="20" t="s">
+      <c r="G37" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H37" s="20"/>
-      <c r="I37" s="20" t="s">
+      <c r="H37" s="16"/>
+      <c r="I37" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="J37" s="20"/>
-      <c r="K37" s="20"/>
-      <c r="L37" s="20" t="s">
-        <v>101</v>
+      <c r="J37" s="16"/>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16" t="s">
+        <v>100</v>
       </c>
       <c r="M37" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2675,35 +2696,35 @@
       <c r="N37" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="O37" s="21" t="s">
-        <v>107</v>
+      <c r="O37" s="18" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="38" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B38" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C38" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C38" s="16"/>
       <c r="D38" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1B</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G38" s="20" t="s">
+      <c r="G38" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H38" s="20"/>
-      <c r="I38" s="20" t="s">
-        <v>138</v>
-      </c>
-      <c r="J38" s="20"/>
-      <c r="K38" s="20"/>
-      <c r="L38" s="20"/>
+      <c r="H38" s="16"/>
+      <c r="I38" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="J38" s="16"/>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16"/>
       <c r="M38" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1B</v>
@@ -2711,13 +2732,13 @@
       <c r="N38" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="21"/>
+      <c r="O38" s="18"/>
     </row>
     <row r="39" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B39" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C39" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C39" s="16"/>
       <c r="D39" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1C</v>
@@ -2732,14 +2753,14 @@
         <v>12</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I39" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I39" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="J39" s="20"/>
-      <c r="K39" s="20"/>
-      <c r="L39" s="20"/>
+      <c r="J39" s="16"/>
+      <c r="K39" s="16"/>
+      <c r="L39" s="16"/>
       <c r="M39" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1C</v>
@@ -2747,11 +2768,11 @@
       <c r="N39" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O39" s="21"/>
+      <c r="O39" s="18"/>
     </row>
     <row r="40" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B40" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>52</v>
@@ -2761,20 +2782,20 @@
         <v>1D</v>
       </c>
       <c r="E40" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F40" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="F40" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20" t="s">
-        <v>144</v>
-      </c>
-      <c r="J40" s="20"/>
-      <c r="K40" s="20"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="16"/>
       <c r="L40" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M40" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2783,15 +2804,15 @@
       <c r="N40" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O40" s="21" t="s">
-        <v>158</v>
+      <c r="O40" s="18" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="41" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B41" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C41" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D41" s="3" t="str">
@@ -2804,17 +2825,17 @@
       <c r="F41" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G41" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="H41" s="20"/>
-      <c r="I41" s="20" t="s">
+      <c r="G41" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="H41" s="16"/>
+      <c r="I41" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="J41" s="20"/>
-      <c r="K41" s="20"/>
+      <c r="J41" s="16"/>
+      <c r="K41" s="16"/>
       <c r="L41" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M41" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2823,14 +2844,14 @@
       <c r="N41" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="O41" s="21"/>
+      <c r="O41" s="18"/>
       <c r="T41" s="2"/>
     </row>
     <row r="42" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B42" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C42" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C42" s="16"/>
       <c r="D42" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1F</v>
@@ -2841,17 +2862,17 @@
       <c r="F42" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G42" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="H42" s="20"/>
-      <c r="I42" s="20" t="s">
+      <c r="G42" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="H42" s="16"/>
+      <c r="I42" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="J42" s="20"/>
-      <c r="K42" s="20"/>
+      <c r="J42" s="16"/>
+      <c r="K42" s="16"/>
       <c r="L42" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M42" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2860,13 +2881,13 @@
       <c r="N42" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="O42" s="21"/>
+      <c r="O42" s="18"/>
     </row>
     <row r="43" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B43" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C43" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C43" s="16" t="s">
         <v>51</v>
       </c>
       <c r="D43" s="3" t="str">
@@ -2879,27 +2900,27 @@
       <c r="F43" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G43" s="20" t="s">
+      <c r="G43" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H43" s="20"/>
-      <c r="I43" s="20" t="s">
+      <c r="H43" s="16"/>
+      <c r="I43" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="J43" s="20"/>
-      <c r="K43" s="20"/>
-      <c r="L43" s="20" t="s">
+      <c r="J43" s="16"/>
+      <c r="K43" s="16"/>
+      <c r="L43" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="M43" s="20"/>
-      <c r="N43" s="20"/>
-      <c r="O43" s="21"/>
+      <c r="M43" s="16"/>
+      <c r="N43" s="16"/>
+      <c r="O43" s="18"/>
     </row>
     <row r="44" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B44" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C44" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C44" s="16"/>
       <c r="D44" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 32))</f>
         <v>40~5F</v>
@@ -2910,31 +2931,31 @@
       <c r="F44" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G44" s="20" t="s">
+      <c r="G44" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H44" s="20"/>
-      <c r="I44" s="20" t="s">
+      <c r="H44" s="16"/>
+      <c r="I44" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="J44" s="20"/>
-      <c r="K44" s="20"/>
+      <c r="J44" s="16"/>
+      <c r="K44" s="16"/>
       <c r="L44" s="6" t="s">
         <v>46</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="N44" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="O44" s="21"/>
+        <v>107</v>
+      </c>
+      <c r="N44" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="O44" s="18"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B45" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C45" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>52</v>
       </c>
       <c r="D45" s="3" t="str">
@@ -2947,67 +2968,67 @@
       <c r="F45" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G45" s="20" t="s">
+      <c r="G45" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H45" s="20"/>
-      <c r="I45" s="20" t="s">
+      <c r="H45" s="16"/>
+      <c r="I45" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="J45" s="20"/>
-      <c r="K45" s="20"/>
+      <c r="J45" s="16"/>
+      <c r="K45" s="16"/>
       <c r="L45" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M45" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="N45" s="20" t="s">
+      <c r="N45" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="O45" s="21"/>
+      <c r="O45" s="18"/>
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B46" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C46" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C46" s="16"/>
       <c r="D46" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 8))</f>
         <v>68~6F</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G46" s="20" t="s">
+      <c r="G46" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H46" s="20"/>
-      <c r="I46" s="20" t="s">
+      <c r="H46" s="16"/>
+      <c r="I46" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="J46" s="20"/>
-      <c r="K46" s="20"/>
+      <c r="J46" s="16"/>
+      <c r="K46" s="16"/>
       <c r="L46" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M46" s="3" t="str">
         <f t="shared" ref="M46:M52" si="5">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M45)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M45)+1))</f>
         <v>01</v>
       </c>
-      <c r="N46" s="20" t="s">
+      <c r="N46" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="O46" s="21"/>
+      <c r="O46" s="18"/>
     </row>
     <row r="47" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B47" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C47" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C47" s="16"/>
       <c r="D47" s="4" t="str">
         <f>DEC2HEX(HEX2DEC(RIGHT(D46,LEN(D46)-FIND("~",D46,1))) + 1)</f>
         <v>70</v>
@@ -3018,32 +3039,32 @@
       <c r="F47" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G47" s="20" t="s">
+      <c r="G47" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H47" s="20"/>
-      <c r="I47" s="20" t="s">
+      <c r="H47" s="16"/>
+      <c r="I47" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="J47" s="20"/>
-      <c r="K47" s="20"/>
+      <c r="J47" s="16"/>
+      <c r="K47" s="16"/>
       <c r="L47" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M47" s="3" t="str">
         <f t="shared" si="5"/>
         <v>02</v>
       </c>
-      <c r="N47" s="20" t="s">
+      <c r="N47" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="O47" s="21"/>
+      <c r="O47" s="18"/>
     </row>
     <row r="48" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B48" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C48" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C48" s="16"/>
       <c r="D48" s="3" t="str">
         <f t="shared" ref="D48:D54" si="6">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D47)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D47)+1))</f>
         <v>71</v>
@@ -3051,135 +3072,135 @@
       <c r="E48" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F48" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G48" s="20"/>
-      <c r="H48" s="20"/>
-      <c r="I48" s="20" t="s">
+      <c r="F48" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G48" s="16"/>
+      <c r="H48" s="16"/>
+      <c r="I48" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="J48" s="20"/>
-      <c r="K48" s="20"/>
+      <c r="J48" s="16"/>
+      <c r="K48" s="16"/>
       <c r="L48" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M48" s="3" t="str">
         <f t="shared" si="5"/>
         <v>03</v>
       </c>
-      <c r="N48" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="O48" s="21"/>
+      <c r="N48" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="O48" s="18"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C49" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C49" s="16"/>
       <c r="D49" s="3" t="str">
         <f t="shared" si="6"/>
         <v>72</v>
       </c>
       <c r="E49" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F49" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G49" s="16"/>
+      <c r="H49" s="16"/>
+      <c r="I49" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="F49" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G49" s="20"/>
-      <c r="H49" s="20"/>
-      <c r="I49" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="J49" s="20"/>
-      <c r="K49" s="20"/>
+      <c r="J49" s="16"/>
+      <c r="K49" s="16"/>
       <c r="L49" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M49" s="3" t="str">
         <f t="shared" si="5"/>
         <v>04</v>
       </c>
-      <c r="N49" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="O49" s="21"/>
+      <c r="N49" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="O49" s="18"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C50" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C50" s="16"/>
       <c r="D50" s="3" t="str">
         <f t="shared" si="6"/>
         <v>73</v>
       </c>
       <c r="E50" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F50" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G50" s="16"/>
+      <c r="H50" s="16"/>
+      <c r="I50" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="F50" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G50" s="20"/>
-      <c r="H50" s="20"/>
-      <c r="I50" s="20" t="s">
-        <v>169</v>
-      </c>
-      <c r="J50" s="20"/>
-      <c r="K50" s="20"/>
+      <c r="J50" s="16"/>
+      <c r="K50" s="16"/>
       <c r="L50" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M50" s="3" t="str">
         <f t="shared" si="5"/>
         <v>05</v>
       </c>
-      <c r="N50" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="O50" s="21"/>
+      <c r="N50" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="O50" s="18"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C51" s="20"/>
+        <v>87</v>
+      </c>
+      <c r="C51" s="16"/>
       <c r="D51" s="3" t="str">
         <f t="shared" si="6"/>
         <v>74</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="F51" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="J51" s="20"/>
-      <c r="K51" s="20"/>
+        <v>156</v>
+      </c>
+      <c r="F51" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G51" s="16"/>
+      <c r="H51" s="16"/>
+      <c r="I51" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="J51" s="16"/>
+      <c r="K51" s="16"/>
       <c r="L51" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M51" s="3" t="str">
         <f t="shared" si="5"/>
         <v>06</v>
       </c>
-      <c r="N51" s="20" t="s">
+      <c r="N51" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="O51" s="21"/>
+      <c r="O51" s="18"/>
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C52" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C52" s="16"/>
       <c r="D52" s="3" t="str">
         <f t="shared" si="6"/>
         <v>75</v>
@@ -3187,33 +3208,33 @@
       <c r="E52" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F52" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="20" t="s">
+      <c r="F52" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G52" s="16"/>
+      <c r="H52" s="16"/>
+      <c r="I52" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="J52" s="20"/>
-      <c r="K52" s="20"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="16"/>
       <c r="L52" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M52" s="3" t="str">
         <f t="shared" si="5"/>
         <v>07</v>
       </c>
-      <c r="N52" s="20" t="s">
+      <c r="N52" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="O52" s="21"/>
+      <c r="O52" s="18"/>
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C53" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C53" s="16" t="s">
         <v>50</v>
       </c>
       <c r="D53" s="3" t="str">
@@ -3221,126 +3242,126 @@
         <v>76</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="F53" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G53" s="20"/>
-      <c r="H53" s="20"/>
-      <c r="I53" s="20" t="s">
-        <v>170</v>
-      </c>
-      <c r="J53" s="20"/>
-      <c r="K53" s="20"/>
+        <v>97</v>
+      </c>
+      <c r="F53" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G53" s="16"/>
+      <c r="H53" s="16"/>
+      <c r="I53" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="J53" s="16"/>
+      <c r="K53" s="16"/>
       <c r="L53" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M53" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(M52) + 1),"~",DEC2HEX(HEX2DEC(M52) + 24))</f>
         <v>8~1F</v>
       </c>
-      <c r="N53" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="O53" s="21"/>
+      <c r="N53" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="O53" s="18"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C54" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C54" s="16"/>
       <c r="D54" s="3" t="str">
         <f t="shared" si="6"/>
         <v>77</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="F54" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="20" t="s">
-        <v>207</v>
-      </c>
-      <c r="J54" s="20"/>
-      <c r="K54" s="20"/>
-      <c r="L54" s="20" t="s">
-        <v>109</v>
-      </c>
-      <c r="M54" s="20"/>
-      <c r="N54" s="20"/>
-      <c r="O54" s="21"/>
+        <v>86</v>
+      </c>
+      <c r="F54" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G54" s="16"/>
+      <c r="H54" s="16"/>
+      <c r="I54" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="J54" s="16"/>
+      <c r="K54" s="16"/>
+      <c r="L54" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="M54" s="16"/>
+      <c r="N54" s="16"/>
+      <c r="O54" s="18"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C55" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C55" s="16"/>
       <c r="D55" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D54)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D54)+1))</f>
         <v>78</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>83</v>
+        <v>203</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>4</v>
+        <v>204</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I55" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="J55" s="20"/>
-      <c r="K55" s="20"/>
+        <v>213</v>
+      </c>
+      <c r="I55" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="J55" s="16"/>
+      <c r="K55" s="16"/>
       <c r="L55" s="5" t="s">
         <v>39</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N55" s="5" t="s">
         <v>39</v>
       </c>
       <c r="O55" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C56" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C56" s="16"/>
       <c r="D56" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D55)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D55)+1))</f>
         <v>79</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>147</v>
+        <v>205</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>91</v>
+        <v>206</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>152</v>
+        <v>207</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I56" s="20" t="s">
-        <v>150</v>
-      </c>
-      <c r="J56" s="20"/>
-      <c r="K56" s="20"/>
+        <v>213</v>
+      </c>
+      <c r="I56" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="J56" s="16"/>
+      <c r="K56" s="16"/>
       <c r="L56" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M56" s="7" t="s">
         <v>27</v>
@@ -3350,14 +3371,14 @@
         <v>4</v>
       </c>
       <c r="O56" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C57" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="C57" s="16" t="s">
         <v>47</v>
       </c>
       <c r="D57" s="3" t="str">
@@ -3365,22 +3386,22 @@
         <v>7A</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="I57" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="J57" s="20"/>
-      <c r="K57" s="20"/>
+        <v>182</v>
+      </c>
+      <c r="I57" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="J57" s="16"/>
+      <c r="K57" s="16"/>
       <c r="L57" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L56+1)</f>
         <v>1</v>
@@ -3393,35 +3414,35 @@
         <v>5</v>
       </c>
       <c r="O57" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B58" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C58" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C58" s="16"/>
       <c r="D58" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D57)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D57)+1))</f>
         <v>7B</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="I58" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="J58" s="20"/>
-      <c r="K58" s="20"/>
+        <v>182</v>
+      </c>
+      <c r="I58" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="J58" s="16"/>
+      <c r="K58" s="16"/>
       <c r="L58" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L57+1)</f>
         <v>2</v>
@@ -3434,14 +3455,14 @@
         <v>6</v>
       </c>
       <c r="O58" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C59" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="C59" s="16" t="s">
         <v>38</v>
       </c>
       <c r="D59" s="3" t="str">
@@ -3449,20 +3470,20 @@
         <v>7C</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="F59" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G59" s="20"/>
+        <v>170</v>
+      </c>
+      <c r="F59" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G59" s="16"/>
       <c r="H59" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="I59" s="20" t="s">
-        <v>178</v>
-      </c>
-      <c r="J59" s="20"/>
-      <c r="K59" s="20"/>
+        <v>171</v>
+      </c>
+      <c r="I59" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="J59" s="16"/>
+      <c r="K59" s="16"/>
       <c r="L59" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L58+1)</f>
         <v>3</v>
@@ -3475,45 +3496,45 @@
         <v>7</v>
       </c>
       <c r="O59" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B60" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C60" s="20"/>
+        <v>88</v>
+      </c>
+      <c r="C60" s="16"/>
       <c r="D60" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7D</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="I60" s="20" t="s">
-        <v>174</v>
-      </c>
-      <c r="J60" s="20"/>
-      <c r="K60" s="20"/>
-      <c r="L60" s="20" t="s">
-        <v>209</v>
-      </c>
-      <c r="M60" s="20"/>
-      <c r="N60" s="20"/>
-      <c r="O60" s="21"/>
+        <v>167</v>
+      </c>
+      <c r="I60" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="J60" s="16"/>
+      <c r="K60" s="16"/>
+      <c r="L60" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="M60" s="16"/>
+      <c r="N60" s="16"/>
+      <c r="O60" s="18"/>
     </row>
     <row r="61" spans="2:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="9" t="s">
-        <v>210</v>
+        <v>88</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>82</v>
@@ -3526,57 +3547,57 @@
         <v>82</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G61" s="13" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="I61" s="20" t="s">
-        <v>191</v>
-      </c>
-      <c r="J61" s="20"/>
-      <c r="K61" s="20"/>
+        <v>159</v>
+      </c>
+      <c r="I61" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="J61" s="16"/>
+      <c r="K61" s="16"/>
       <c r="L61" s="15" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="M61" s="15"/>
       <c r="N61" s="15"/>
-      <c r="O61" s="16"/>
+      <c r="O61" s="29"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7F</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="F62" s="20" t="s">
-        <v>194</v>
-      </c>
-      <c r="G62" s="20"/>
+        <v>186</v>
+      </c>
+      <c r="F62" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="G62" s="16"/>
       <c r="H62" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="I62" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="J62" s="20"/>
-      <c r="K62" s="20"/>
+        <v>187</v>
+      </c>
+      <c r="I62" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="J62" s="16"/>
+      <c r="K62" s="16"/>
       <c r="L62" s="4" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="M62" s="3" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="N62" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L67,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L67,"-", -1))+1,"0"))</f>
@@ -3586,34 +3607,34 @@
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(D62) + 1),"~","FF")</f>
         <v>80~FF</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="F63" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="G63" s="20"/>
-      <c r="H63" s="20"/>
-      <c r="I63" s="20" t="s">
-        <v>180</v>
-      </c>
-      <c r="J63" s="20"/>
-      <c r="K63" s="20"/>
+        <v>83</v>
+      </c>
+      <c r="F63" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G63" s="16"/>
+      <c r="H63" s="16"/>
+      <c r="I63" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="J63" s="16"/>
+      <c r="K63" s="16"/>
       <c r="L63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L62,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L62,"-", -1))+1,"0"))</f>
         <v>ex-1</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="N63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N62,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N62,"-", -1))+1,"0"))</f>
@@ -3622,32 +3643,34 @@
       <c r="O63" s="10"/>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B64" s="17" t="s">
-        <v>181</v>
+      <c r="B64" s="30" t="s">
+        <v>175</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="G64" s="20"/>
-      <c r="H64" s="20"/>
-      <c r="I64" s="20"/>
-      <c r="J64" s="20"/>
-      <c r="K64" s="20"/>
+        <v>177</v>
+      </c>
+      <c r="G64" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="H64" s="16"/>
+      <c r="I64" s="32"/>
+      <c r="J64" s="32"/>
+      <c r="K64" s="32"/>
       <c r="L64" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L63,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L63,"-", -1))+1,"0"))</f>
         <v>ex-2</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="N64" s="3" t="str">
         <f t="shared" ref="N64:N67" si="8">_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(N63,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(N63,"-", -1))+1,"0"))</f>
@@ -3656,30 +3679,32 @@
       <c r="O64" s="10"/>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B65" s="17"/>
+      <c r="B65" s="30"/>
       <c r="C65" s="3" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="G65" s="20"/>
-      <c r="H65" s="20"/>
-      <c r="I65" s="20"/>
-      <c r="J65" s="20"/>
-      <c r="K65" s="20"/>
+        <v>180</v>
+      </c>
+      <c r="G65" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="H65" s="16"/>
+      <c r="I65" s="32"/>
+      <c r="J65" s="32"/>
+      <c r="K65" s="32"/>
       <c r="L65" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L64,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L64,"-", -1))+1,"0"))</f>
         <v>ex-3</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="N65" s="3" t="str">
         <f t="shared" si="8"/>
@@ -3688,24 +3713,26 @@
       <c r="O65" s="10"/>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B66" s="17"/>
+      <c r="B66" s="30"/>
       <c r="C66" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="D66" s="20"/>
-      <c r="E66" s="20"/>
-      <c r="F66" s="20"/>
-      <c r="G66" s="20"/>
-      <c r="H66" s="20"/>
-      <c r="I66" s="20"/>
-      <c r="J66" s="20"/>
-      <c r="K66" s="20"/>
+        <v>191</v>
+      </c>
+      <c r="D66" s="16"/>
+      <c r="E66" s="16"/>
+      <c r="F66" s="16"/>
+      <c r="G66" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="H66" s="16"/>
+      <c r="I66" s="32"/>
+      <c r="J66" s="32"/>
+      <c r="K66" s="32"/>
       <c r="L66" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L65,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L65,"-", -1))+1,"0"))</f>
         <v>ex-4</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="N66" s="3" t="str">
         <f t="shared" si="8"/>
@@ -3714,22 +3741,24 @@
       <c r="O66" s="10"/>
     </row>
     <row r="67" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B67" s="18"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="31"/>
-      <c r="E67" s="31"/>
-      <c r="F67" s="31"/>
-      <c r="G67" s="31"/>
-      <c r="H67" s="31"/>
-      <c r="I67" s="31"/>
-      <c r="J67" s="31"/>
-      <c r="K67" s="31"/>
+      <c r="B67" s="31"/>
+      <c r="C67" s="17"/>
+      <c r="D67" s="17"/>
+      <c r="E67" s="17"/>
+      <c r="F67" s="17"/>
+      <c r="G67" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="H67" s="17"/>
+      <c r="I67" s="33"/>
+      <c r="J67" s="33"/>
+      <c r="K67" s="33"/>
       <c r="L67" s="12" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(L66,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(L66,"-", -1))+1,"0"))</f>
         <v>ex-5</v>
       </c>
       <c r="M67" s="12" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="N67" s="12" t="str">
         <f t="shared" si="8"/>
@@ -3738,30 +3767,91 @@
       <c r="O67" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="128">
-    <mergeCell ref="C66:F67"/>
-    <mergeCell ref="G64:K67"/>
-    <mergeCell ref="I61:K61"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="O40:O42"/>
-    <mergeCell ref="F63:H63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="N53:O53"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="L54:O54"/>
-    <mergeCell ref="F54:H54"/>
-    <mergeCell ref="L60:O60"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="N46:O46"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="N48:O48"/>
-    <mergeCell ref="N49:O49"/>
+  <mergeCells count="131">
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="L61:O61"/>
+    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="AF15:AG15"/>
+    <mergeCell ref="L43:O43"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="I49:K49"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="U15:AB15"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="C11:C36"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="N44:O44"/>
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:K46"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="O37:O39"/>
+    <mergeCell ref="L11:L36"/>
+    <mergeCell ref="O13:O15"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="O33:O34"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="C45:C52"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="F51:H51"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="C43:C44"/>
     <mergeCell ref="C37:C39"/>
     <mergeCell ref="I51:K51"/>
     <mergeCell ref="F53:H53"/>
@@ -3786,87 +3876,29 @@
     <mergeCell ref="I54:K54"/>
     <mergeCell ref="I58:K58"/>
     <mergeCell ref="C41:C42"/>
+    <mergeCell ref="C66:F67"/>
+    <mergeCell ref="I61:K61"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="O40:O42"/>
+    <mergeCell ref="F63:H63"/>
+    <mergeCell ref="I63:K63"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="N53:O53"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="I59:K59"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="L54:O54"/>
+    <mergeCell ref="F54:H54"/>
+    <mergeCell ref="L60:O60"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="N46:O46"/>
+    <mergeCell ref="N47:O47"/>
+    <mergeCell ref="N48:O48"/>
+    <mergeCell ref="N49:O49"/>
     <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="C45:C52"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="N44:O44"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="O37:O39"/>
-    <mergeCell ref="L11:L36"/>
-    <mergeCell ref="O13:O15"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="O33:O34"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="L61:O61"/>
-    <mergeCell ref="B64:B67"/>
-    <mergeCell ref="AF15:AG15"/>
-    <mergeCell ref="L43:O43"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="T34:V34"/>
-    <mergeCell ref="W34:Y34"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="U15:AB15"/>
-    <mergeCell ref="I55:K55"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>